<commit_message>
Expand template with all common required/optional fields + rollback
Template now covers:
- Campaign: buying_type (AUCTION/RESERVED)
- Ad set: bid_strategy, bid_amount_usd, destination_type, start_time,
  end_time, pixel_id + custom_event_type (promoted_object for
  conversions)
- Ad: instagram_actor_id, url_tags (UTM)

Uploader applies these conditionally so existing simple uploads still
work. On failure during a real upload, the script now deletes the
entities it just created (ads, then ad sets, then campaigns) so users
don't have to manually clean up orphans in Ads Manager.
</commit_message>
<xml_diff>
--- a/template.xlsx
+++ b/template.xlsx
@@ -413,28 +413,38 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S2"/>
+  <dimension ref="A1:AC2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="1"/>
     <col width="20" customWidth="1" min="2" max="2"/>
-    <col width="23" customWidth="1" min="3" max="3"/>
-    <col width="14" customWidth="1" min="4" max="4"/>
-    <col width="18" customWidth="1" min="5" max="5"/>
-    <col width="15" customWidth="1" min="6" max="6"/>
-    <col width="19" customWidth="1" min="7" max="7"/>
-    <col width="19" customWidth="1" min="8" max="8"/>
-    <col width="14" customWidth="1" min="9" max="9"/>
-    <col width="14" customWidth="1" min="10" max="10"/>
-    <col width="14" customWidth="1" min="11" max="11"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="23" customWidth="1" min="4" max="4"/>
+    <col width="14" customWidth="1" min="5" max="5"/>
+    <col width="18" customWidth="1" min="6" max="6"/>
+    <col width="14" customWidth="1" min="7" max="7"/>
+    <col width="16" customWidth="1" min="8" max="8"/>
+    <col width="15" customWidth="1" min="9" max="9"/>
+    <col width="19" customWidth="1" min="10" max="10"/>
+    <col width="18" customWidth="1" min="11" max="11"/>
     <col width="14" customWidth="1" min="12" max="12"/>
     <col width="14" customWidth="1" min="13" max="13"/>
     <col width="14" customWidth="1" min="14" max="14"/>
-    <col width="14" customWidth="1" min="15" max="15"/>
-    <col width="14" customWidth="1" min="16" max="16"/>
+    <col width="19" customWidth="1" min="15" max="15"/>
+    <col width="19" customWidth="1" min="16" max="16"/>
     <col width="14" customWidth="1" min="17" max="17"/>
     <col width="14" customWidth="1" min="18" max="18"/>
     <col width="14" customWidth="1" min="19" max="19"/>
+    <col width="14" customWidth="1" min="20" max="20"/>
+    <col width="20" customWidth="1" min="21" max="21"/>
+    <col width="14" customWidth="1" min="22" max="22"/>
+    <col width="14" customWidth="1" min="23" max="23"/>
+    <col width="14" customWidth="1" min="24" max="24"/>
+    <col width="14" customWidth="1" min="25" max="25"/>
+    <col width="14" customWidth="1" min="26" max="26"/>
+    <col width="14" customWidth="1" min="27" max="27"/>
+    <col width="14" customWidth="1" min="28" max="28"/>
+    <col width="14" customWidth="1" min="29" max="29"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -450,85 +460,135 @@
       </c>
       <c r="C1" t="inlineStr">
         <is>
+          <t>buying_type</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
           <t>special_ad_categories</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>adset_name</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>daily_budget_usd</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>bid_strategy</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>bid_amount_usd</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
         <is>
           <t>billing_event</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="J1" t="inlineStr">
         <is>
           <t>optimization_goal</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="K1" t="inlineStr">
+        <is>
+          <t>destination_type</t>
+        </is>
+      </c>
+      <c r="L1" t="inlineStr">
+        <is>
+          <t>start_time</t>
+        </is>
+      </c>
+      <c r="M1" t="inlineStr">
+        <is>
+          <t>end_time</t>
+        </is>
+      </c>
+      <c r="N1" t="inlineStr">
+        <is>
+          <t>pixel_id</t>
+        </is>
+      </c>
+      <c r="O1" t="inlineStr">
+        <is>
+          <t>custom_event_type</t>
+        </is>
+      </c>
+      <c r="P1" t="inlineStr">
         <is>
           <t>saved_audience_id</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
+      <c r="Q1" t="inlineStr">
         <is>
           <t>countries</t>
         </is>
       </c>
-      <c r="J1" t="inlineStr">
+      <c r="R1" t="inlineStr">
         <is>
           <t>age_min</t>
         </is>
       </c>
-      <c r="K1" t="inlineStr">
+      <c r="S1" t="inlineStr">
         <is>
           <t>age_max</t>
         </is>
       </c>
-      <c r="L1" t="inlineStr">
+      <c r="T1" t="inlineStr">
         <is>
           <t>page_id</t>
         </is>
       </c>
-      <c r="M1" t="inlineStr">
+      <c r="U1" t="inlineStr">
+        <is>
+          <t>instagram_actor_id</t>
+        </is>
+      </c>
+      <c r="V1" t="inlineStr">
         <is>
           <t>ad_name</t>
         </is>
       </c>
-      <c r="N1" t="inlineStr">
+      <c r="W1" t="inlineStr">
         <is>
           <t>image_url</t>
         </is>
       </c>
-      <c r="O1" t="inlineStr">
+      <c r="X1" t="inlineStr">
         <is>
           <t>primary_text</t>
         </is>
       </c>
-      <c r="P1" t="inlineStr">
+      <c r="Y1" t="inlineStr">
         <is>
           <t>headline</t>
         </is>
       </c>
-      <c r="Q1" t="inlineStr">
+      <c r="Z1" t="inlineStr">
         <is>
           <t>description</t>
         </is>
       </c>
-      <c r="R1" t="inlineStr">
+      <c r="AA1" t="inlineStr">
         <is>
           <t>link_url</t>
         </is>
       </c>
-      <c r="S1" t="inlineStr">
+      <c r="AB1" t="inlineStr">
+        <is>
+          <t>url_tags</t>
+        </is>
+      </c>
+      <c r="AC1" t="inlineStr">
         <is>
           <t>cta</t>
         </is>
@@ -547,95 +607,133 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
+          <t>AUCTION</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
           <t>NONE</t>
         </is>
       </c>
-      <c r="D2" t="inlineStr">
+      <c r="E2" t="inlineStr">
         <is>
           <t>US Broad 25-54</t>
         </is>
       </c>
-      <c r="E2" t="n">
+      <c r="F2" t="n">
         <v>50</v>
       </c>
-      <c r="F2" t="inlineStr">
-        <is>
-          <t>IMPRESSIONS</t>
-        </is>
-      </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>LINK_CLICKS</t>
+          <t>LOWEST_COST_WITHOUT_CAP</t>
         </is>
       </c>
       <c r="H2" t="inlineStr"/>
       <c r="I2" t="inlineStr">
         <is>
+          <t>IMPRESSIONS</t>
+        </is>
+      </c>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>LANDING_PAGE_VIEWS</t>
+        </is>
+      </c>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>WEBSITE</t>
+        </is>
+      </c>
+      <c r="L2" t="inlineStr"/>
+      <c r="M2" t="inlineStr"/>
+      <c r="N2" t="inlineStr"/>
+      <c r="O2" t="inlineStr"/>
+      <c r="P2" t="inlineStr"/>
+      <c r="Q2" t="inlineStr">
+        <is>
           <t>US</t>
         </is>
       </c>
-      <c r="J2" t="n">
+      <c r="R2" t="n">
         <v>25</v>
       </c>
-      <c r="K2" t="n">
+      <c r="S2" t="n">
         <v>54</v>
       </c>
-      <c r="L2" t="inlineStr">
+      <c r="T2" t="inlineStr">
         <is>
           <t>1234567890</t>
         </is>
       </c>
-      <c r="M2" t="inlineStr">
+      <c r="U2" t="inlineStr"/>
+      <c r="V2" t="inlineStr">
         <is>
           <t>Ad A - Static</t>
         </is>
       </c>
-      <c r="N2" t="inlineStr">
+      <c r="W2" t="inlineStr">
         <is>
           <t>https://example.com/creative-a.jpg</t>
         </is>
       </c>
-      <c r="O2" t="inlineStr">
+      <c r="X2" t="inlineStr">
         <is>
           <t>Discover our new spring collection.</t>
         </is>
       </c>
-      <c r="P2" t="inlineStr">
+      <c r="Y2" t="inlineStr">
         <is>
           <t>Spring is here</t>
         </is>
       </c>
-      <c r="Q2" t="inlineStr">
+      <c r="Z2" t="inlineStr">
         <is>
           <t>Shop the drop</t>
         </is>
       </c>
-      <c r="R2" t="inlineStr">
+      <c r="AA2" t="inlineStr">
         <is>
           <t>https://example.com/spring</t>
         </is>
       </c>
-      <c r="S2" t="inlineStr">
+      <c r="AB2" t="inlineStr">
+        <is>
+          <t>utm_source=facebook&amp;utm_medium=cpc&amp;utm_campaign=spring</t>
+        </is>
+      </c>
+      <c r="AC2" t="inlineStr">
         <is>
           <t>SHOP_NOW</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <dataValidations count="5">
+  <dataValidations count="9">
     <dataValidation sqref="B2:B500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid value" error="Pick a valid campaign_objective" promptTitle="campaign_objective" prompt="Choose from the list" type="list">
       <formula1>"OUTCOME_AWARENESS,OUTCOME_TRAFFIC,OUTCOME_ENGAGEMENT,OUTCOME_LEADS,OUTCOME_APP_PROMOTION,OUTCOME_SALES"</formula1>
     </dataValidation>
-    <dataValidation sqref="C2:C500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid value" error="Pick a valid special_ad_categories" promptTitle="special_ad_categories" prompt="Choose from the list" type="list">
+    <dataValidation sqref="C2:C500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid value" error="Pick a valid buying_type" promptTitle="buying_type" prompt="Choose from the list" type="list">
+      <formula1>"AUCTION,RESERVED"</formula1>
+    </dataValidation>
+    <dataValidation sqref="D2:D500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid value" error="Pick a valid special_ad_categories" promptTitle="special_ad_categories" prompt="Choose from the list" type="list">
       <formula1>"NONE,HOUSING,CREDIT,EMPLOYMENT,ISSUES_ELECTIONS_POLITICS,ONLINE_GAMBLING_AND_GAMING,FINANCIAL_PRODUCTS_SERVICES"</formula1>
     </dataValidation>
-    <dataValidation sqref="F2:F500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid value" error="Pick a valid billing_event" promptTitle="billing_event" prompt="Choose from the list" type="list">
+    <dataValidation sqref="G2:G500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid value" error="Pick a valid bid_strategy" promptTitle="bid_strategy" prompt="Choose from the list" type="list">
+      <formula1>"LOWEST_COST_WITHOUT_CAP,LOWEST_COST_WITH_BID_CAP,COST_CAP,LOWEST_COST_WITH_MIN_ROAS"</formula1>
+    </dataValidation>
+    <dataValidation sqref="I2:I500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid value" error="Pick a valid billing_event" promptTitle="billing_event" prompt="Choose from the list" type="list">
       <formula1>"IMPRESSIONS,LINK_CLICKS,POST_ENGAGEMENT,VIDEO_VIEWS,THRUPLAY"</formula1>
     </dataValidation>
-    <dataValidation sqref="G2:G500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid value" error="Pick a valid optimization_goal" promptTitle="optimization_goal" prompt="Choose from the list" type="list">
+    <dataValidation sqref="J2:J500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid value" error="Pick a valid optimization_goal" promptTitle="optimization_goal" prompt="Choose from the list" type="list">
       <formula1>"REACH,IMPRESSIONS,LINK_CLICKS,LANDING_PAGE_VIEWS,POST_ENGAGEMENT,PAGE_LIKES,VIDEO_VIEWS,THRUPLAY,OFFSITE_CONVERSIONS,VALUE,LEAD_GENERATION,QUALITY_LEAD,CONVERSATIONS,APP_INSTALLS,AD_RECALL_LIFT"</formula1>
     </dataValidation>
-    <dataValidation sqref="S2:S500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid value" error="Pick a valid cta" promptTitle="cta" prompt="Choose from the list" type="list">
+    <dataValidation sqref="K2:K500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid value" error="Pick a valid destination_type" promptTitle="destination_type" prompt="Choose from the list" type="list">
+      <formula1>"WEBSITE,APP,MESSENGER,INSTAGRAM_DIRECT,WHATSAPP,FACEBOOK,ON_AD,ON_POST,ON_PAGE,ON_EVENT,ON_VIDEO,SHOP_AUTOMATIC"</formula1>
+    </dataValidation>
+    <dataValidation sqref="O2:O500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid value" error="Pick a valid custom_event_type" promptTitle="custom_event_type" prompt="Choose from the list" type="list">
+      <formula1>",PURCHASE,LEAD,COMPLETE_REGISTRATION,ADD_TO_CART,INITIATE_CHECKOUT,ADD_PAYMENT_INFO,VIEW_CONTENT,SEARCH,SUBSCRIBE,CONTACT,DONATE,OTHER"</formula1>
+    </dataValidation>
+    <dataValidation sqref="AC2:AC500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid value" error="Pick a valid cta" promptTitle="cta" prompt="Choose from the list" type="list">
       <formula1>"SHOP_NOW,LEARN_MORE,SIGN_UP,SUBSCRIBE,DOWNLOAD,BOOK_TRAVEL,CONTACT_US,GET_OFFER,GET_QUOTE,APPLY_NOW,ORDER_NOW,DONATE_NOW,INSTALL_APP,USE_APP,WATCH_MORE,LISTEN_NOW,SEND_MESSAGE,MESSAGE_PAGE,GET_DIRECTIONS,CALL_NOW,NO_BUTTON"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
Expand template with CBO, lifetime budgets, video ads, and more targeting
Adds 20 new columns covering CBO budgets and bidding, campaign schedule,
ad-set lifetime budget / spend caps / pacing / ROAS floor, app-promotion
promoted_object fields, DSA fields, gender + custom-audience targeting,
video ads, and conversion_domain. Guards reject mixed CBO/ABO budgets.
</commit_message>
<xml_diff>
--- a/template.xlsx
+++ b/template.xlsx
@@ -413,38 +413,58 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AC2"/>
+  <dimension ref="A1:AW2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="1"/>
     <col width="20" customWidth="1" min="2" max="2"/>
     <col width="14" customWidth="1" min="3" max="3"/>
     <col width="23" customWidth="1" min="4" max="4"/>
-    <col width="14" customWidth="1" min="5" max="5"/>
-    <col width="18" customWidth="1" min="6" max="6"/>
-    <col width="14" customWidth="1" min="7" max="7"/>
-    <col width="16" customWidth="1" min="8" max="8"/>
-    <col width="15" customWidth="1" min="9" max="9"/>
-    <col width="19" customWidth="1" min="10" max="10"/>
-    <col width="18" customWidth="1" min="11" max="11"/>
-    <col width="14" customWidth="1" min="12" max="12"/>
-    <col width="14" customWidth="1" min="13" max="13"/>
+    <col width="27" customWidth="1" min="5" max="5"/>
+    <col width="30" customWidth="1" min="6" max="6"/>
+    <col width="23" customWidth="1" min="7" max="7"/>
+    <col width="24" customWidth="1" min="8" max="8"/>
+    <col width="21" customWidth="1" min="9" max="9"/>
+    <col width="20" customWidth="1" min="10" max="10"/>
+    <col width="14" customWidth="1" min="11" max="11"/>
+    <col width="18" customWidth="1" min="12" max="12"/>
+    <col width="21" customWidth="1" min="13" max="13"/>
     <col width="14" customWidth="1" min="14" max="14"/>
-    <col width="19" customWidth="1" min="15" max="15"/>
-    <col width="19" customWidth="1" min="16" max="16"/>
-    <col width="14" customWidth="1" min="17" max="17"/>
-    <col width="14" customWidth="1" min="18" max="18"/>
+    <col width="16" customWidth="1" min="15" max="15"/>
+    <col width="16" customWidth="1" min="16" max="16"/>
+    <col width="21" customWidth="1" min="17" max="17"/>
+    <col width="24" customWidth="1" min="18" max="18"/>
     <col width="14" customWidth="1" min="19" max="19"/>
-    <col width="14" customWidth="1" min="20" max="20"/>
-    <col width="20" customWidth="1" min="21" max="21"/>
-    <col width="14" customWidth="1" min="22" max="22"/>
+    <col width="15" customWidth="1" min="20" max="20"/>
+    <col width="19" customWidth="1" min="21" max="21"/>
+    <col width="18" customWidth="1" min="22" max="22"/>
     <col width="14" customWidth="1" min="23" max="23"/>
     <col width="14" customWidth="1" min="24" max="24"/>
     <col width="14" customWidth="1" min="25" max="25"/>
-    <col width="14" customWidth="1" min="26" max="26"/>
-    <col width="14" customWidth="1" min="27" max="27"/>
-    <col width="14" customWidth="1" min="28" max="28"/>
-    <col width="14" customWidth="1" min="29" max="29"/>
+    <col width="19" customWidth="1" min="26" max="26"/>
+    <col width="16" customWidth="1" min="27" max="27"/>
+    <col width="18" customWidth="1" min="28" max="28"/>
+    <col width="17" customWidth="1" min="29" max="29"/>
+    <col width="14" customWidth="1" min="30" max="30"/>
+    <col width="19" customWidth="1" min="31" max="31"/>
+    <col width="14" customWidth="1" min="32" max="32"/>
+    <col width="14" customWidth="1" min="33" max="33"/>
+    <col width="14" customWidth="1" min="34" max="34"/>
+    <col width="14" customWidth="1" min="35" max="35"/>
+    <col width="30" customWidth="1" min="36" max="36"/>
+    <col width="30" customWidth="1" min="37" max="37"/>
+    <col width="14" customWidth="1" min="38" max="38"/>
+    <col width="20" customWidth="1" min="39" max="39"/>
+    <col width="14" customWidth="1" min="40" max="40"/>
+    <col width="14" customWidth="1" min="41" max="41"/>
+    <col width="14" customWidth="1" min="42" max="42"/>
+    <col width="14" customWidth="1" min="43" max="43"/>
+    <col width="14" customWidth="1" min="44" max="44"/>
+    <col width="14" customWidth="1" min="45" max="45"/>
+    <col width="14" customWidth="1" min="46" max="46"/>
+    <col width="14" customWidth="1" min="47" max="47"/>
+    <col width="14" customWidth="1" min="48" max="48"/>
+    <col width="19" customWidth="1" min="49" max="49"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -470,127 +490,227 @@
       </c>
       <c r="E1" t="inlineStr">
         <is>
+          <t>campaign_daily_budget_usd</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>campaign_lifetime_budget_usd</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>campaign_bid_strategy</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>campaign_spend_cap_usd</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>campaign_start_time</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>campaign_stop_time</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr">
+        <is>
           <t>adset_name</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="L1" t="inlineStr">
         <is>
           <t>daily_budget_usd</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="M1" t="inlineStr">
+        <is>
+          <t>lifetime_budget_usd</t>
+        </is>
+      </c>
+      <c r="N1" t="inlineStr">
         <is>
           <t>bid_strategy</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="O1" t="inlineStr">
         <is>
           <t>bid_amount_usd</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
+      <c r="P1" t="inlineStr">
+        <is>
+          <t>bid_roas_floor</t>
+        </is>
+      </c>
+      <c r="Q1" t="inlineStr">
+        <is>
+          <t>daily_spend_cap_usd</t>
+        </is>
+      </c>
+      <c r="R1" t="inlineStr">
+        <is>
+          <t>lifetime_spend_cap_usd</t>
+        </is>
+      </c>
+      <c r="S1" t="inlineStr">
+        <is>
+          <t>pacing_type</t>
+        </is>
+      </c>
+      <c r="T1" t="inlineStr">
         <is>
           <t>billing_event</t>
         </is>
       </c>
-      <c r="J1" t="inlineStr">
+      <c r="U1" t="inlineStr">
         <is>
           <t>optimization_goal</t>
         </is>
       </c>
-      <c r="K1" t="inlineStr">
+      <c r="V1" t="inlineStr">
         <is>
           <t>destination_type</t>
         </is>
       </c>
-      <c r="L1" t="inlineStr">
+      <c r="W1" t="inlineStr">
         <is>
           <t>start_time</t>
         </is>
       </c>
-      <c r="M1" t="inlineStr">
+      <c r="X1" t="inlineStr">
         <is>
           <t>end_time</t>
         </is>
       </c>
-      <c r="N1" t="inlineStr">
+      <c r="Y1" t="inlineStr">
         <is>
           <t>pixel_id</t>
         </is>
       </c>
-      <c r="O1" t="inlineStr">
+      <c r="Z1" t="inlineStr">
         <is>
           <t>custom_event_type</t>
         </is>
       </c>
-      <c r="P1" t="inlineStr">
+      <c r="AA1" t="inlineStr">
+        <is>
+          <t>application_id</t>
+        </is>
+      </c>
+      <c r="AB1" t="inlineStr">
+        <is>
+          <t>object_store_url</t>
+        </is>
+      </c>
+      <c r="AC1" t="inlineStr">
+        <is>
+          <t>dsa_beneficiary</t>
+        </is>
+      </c>
+      <c r="AD1" t="inlineStr">
+        <is>
+          <t>dsa_payor</t>
+        </is>
+      </c>
+      <c r="AE1" t="inlineStr">
         <is>
           <t>saved_audience_id</t>
         </is>
       </c>
-      <c r="Q1" t="inlineStr">
+      <c r="AF1" t="inlineStr">
         <is>
           <t>countries</t>
         </is>
       </c>
-      <c r="R1" t="inlineStr">
+      <c r="AG1" t="inlineStr">
         <is>
           <t>age_min</t>
         </is>
       </c>
-      <c r="S1" t="inlineStr">
+      <c r="AH1" t="inlineStr">
         <is>
           <t>age_max</t>
         </is>
       </c>
-      <c r="T1" t="inlineStr">
+      <c r="AI1" t="inlineStr">
+        <is>
+          <t>genders</t>
+        </is>
+      </c>
+      <c r="AJ1" t="inlineStr">
+        <is>
+          <t>included_custom_audience_ids</t>
+        </is>
+      </c>
+      <c r="AK1" t="inlineStr">
+        <is>
+          <t>excluded_custom_audience_ids</t>
+        </is>
+      </c>
+      <c r="AL1" t="inlineStr">
         <is>
           <t>page_id</t>
         </is>
       </c>
-      <c r="U1" t="inlineStr">
+      <c r="AM1" t="inlineStr">
         <is>
           <t>instagram_actor_id</t>
         </is>
       </c>
-      <c r="V1" t="inlineStr">
+      <c r="AN1" t="inlineStr">
         <is>
           <t>ad_name</t>
         </is>
       </c>
-      <c r="W1" t="inlineStr">
+      <c r="AO1" t="inlineStr">
         <is>
           <t>image_url</t>
         </is>
       </c>
-      <c r="X1" t="inlineStr">
+      <c r="AP1" t="inlineStr">
+        <is>
+          <t>video_id</t>
+        </is>
+      </c>
+      <c r="AQ1" t="inlineStr">
         <is>
           <t>primary_text</t>
         </is>
       </c>
-      <c r="Y1" t="inlineStr">
+      <c r="AR1" t="inlineStr">
         <is>
           <t>headline</t>
         </is>
       </c>
-      <c r="Z1" t="inlineStr">
+      <c r="AS1" t="inlineStr">
         <is>
           <t>description</t>
         </is>
       </c>
-      <c r="AA1" t="inlineStr">
+      <c r="AT1" t="inlineStr">
         <is>
           <t>link_url</t>
         </is>
       </c>
-      <c r="AB1" t="inlineStr">
+      <c r="AU1" t="inlineStr">
         <is>
           <t>url_tags</t>
         </is>
       </c>
-      <c r="AC1" t="inlineStr">
+      <c r="AV1" t="inlineStr">
         <is>
           <t>cta</t>
+        </is>
+      </c>
+      <c r="AW1" t="inlineStr">
+        <is>
+          <t>conversion_domain</t>
         </is>
       </c>
     </row>
@@ -615,100 +735,124 @@
           <t>NONE</t>
         </is>
       </c>
-      <c r="E2" t="inlineStr">
+      <c r="E2" t="inlineStr"/>
+      <c r="F2" t="inlineStr"/>
+      <c r="G2" t="inlineStr"/>
+      <c r="H2" t="inlineStr"/>
+      <c r="I2" t="inlineStr"/>
+      <c r="J2" t="inlineStr"/>
+      <c r="K2" t="inlineStr">
         <is>
           <t>US Broad 25-54</t>
         </is>
       </c>
-      <c r="F2" t="n">
+      <c r="L2" t="n">
         <v>50</v>
       </c>
-      <c r="G2" t="inlineStr">
+      <c r="M2" t="inlineStr"/>
+      <c r="N2" t="inlineStr">
         <is>
           <t>LOWEST_COST_WITHOUT_CAP</t>
         </is>
       </c>
-      <c r="H2" t="inlineStr"/>
-      <c r="I2" t="inlineStr">
-        <is>
-          <t>IMPRESSIONS</t>
-        </is>
-      </c>
-      <c r="J2" t="inlineStr">
-        <is>
-          <t>LANDING_PAGE_VIEWS</t>
-        </is>
-      </c>
-      <c r="K2" t="inlineStr">
-        <is>
-          <t>WEBSITE</t>
-        </is>
-      </c>
-      <c r="L2" t="inlineStr"/>
-      <c r="M2" t="inlineStr"/>
-      <c r="N2" t="inlineStr"/>
       <c r="O2" t="inlineStr"/>
       <c r="P2" t="inlineStr"/>
-      <c r="Q2" t="inlineStr">
+      <c r="Q2" t="inlineStr"/>
+      <c r="R2" t="inlineStr"/>
+      <c r="S2" t="inlineStr"/>
+      <c r="T2" t="inlineStr">
+        <is>
+          <t>IMPRESSIONS</t>
+        </is>
+      </c>
+      <c r="U2" t="inlineStr">
+        <is>
+          <t>LANDING_PAGE_VIEWS</t>
+        </is>
+      </c>
+      <c r="V2" t="inlineStr">
+        <is>
+          <t>WEBSITE</t>
+        </is>
+      </c>
+      <c r="W2" t="inlineStr"/>
+      <c r="X2" t="inlineStr"/>
+      <c r="Y2" t="inlineStr"/>
+      <c r="Z2" t="inlineStr"/>
+      <c r="AA2" t="inlineStr"/>
+      <c r="AB2" t="inlineStr"/>
+      <c r="AC2" t="inlineStr"/>
+      <c r="AD2" t="inlineStr"/>
+      <c r="AE2" t="inlineStr"/>
+      <c r="AF2" t="inlineStr">
         <is>
           <t>US</t>
         </is>
       </c>
-      <c r="R2" t="n">
+      <c r="AG2" t="n">
         <v>25</v>
       </c>
-      <c r="S2" t="n">
+      <c r="AH2" t="n">
         <v>54</v>
       </c>
-      <c r="T2" t="inlineStr">
+      <c r="AI2" t="inlineStr"/>
+      <c r="AJ2" t="inlineStr"/>
+      <c r="AK2" t="inlineStr"/>
+      <c r="AL2" t="inlineStr">
         <is>
           <t>1234567890</t>
         </is>
       </c>
-      <c r="U2" t="inlineStr"/>
-      <c r="V2" t="inlineStr">
+      <c r="AM2" t="inlineStr"/>
+      <c r="AN2" t="inlineStr">
         <is>
           <t>Ad A - Static</t>
         </is>
       </c>
-      <c r="W2" t="inlineStr">
+      <c r="AO2" t="inlineStr">
         <is>
           <t>https://example.com/creative-a.jpg</t>
         </is>
       </c>
-      <c r="X2" t="inlineStr">
+      <c r="AP2" t="inlineStr"/>
+      <c r="AQ2" t="inlineStr">
         <is>
           <t>Discover our new spring collection.</t>
         </is>
       </c>
-      <c r="Y2" t="inlineStr">
+      <c r="AR2" t="inlineStr">
         <is>
           <t>Spring is here</t>
         </is>
       </c>
-      <c r="Z2" t="inlineStr">
+      <c r="AS2" t="inlineStr">
         <is>
           <t>Shop the drop</t>
         </is>
       </c>
-      <c r="AA2" t="inlineStr">
+      <c r="AT2" t="inlineStr">
         <is>
           <t>https://example.com/spring</t>
         </is>
       </c>
-      <c r="AB2" t="inlineStr">
+      <c r="AU2" t="inlineStr">
         <is>
           <t>utm_source=facebook&amp;utm_medium=cpc&amp;utm_campaign=spring</t>
         </is>
       </c>
-      <c r="AC2" t="inlineStr">
+      <c r="AV2" t="inlineStr">
         <is>
           <t>SHOP_NOW</t>
+        </is>
+      </c>
+      <c r="AW2" t="inlineStr">
+        <is>
+          <t>example.com</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <dataValidations count="9">
+  <dataValidations count="12">
     <dataValidation sqref="B2:B500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid value" error="Pick a valid campaign_objective" promptTitle="campaign_objective" prompt="Choose from the list" type="list">
       <formula1>"OUTCOME_AWARENESS,OUTCOME_TRAFFIC,OUTCOME_ENGAGEMENT,OUTCOME_LEADS,OUTCOME_APP_PROMOTION,OUTCOME_SALES"</formula1>
     </dataValidation>
@@ -718,22 +862,31 @@
     <dataValidation sqref="D2:D500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid value" error="Pick a valid special_ad_categories" promptTitle="special_ad_categories" prompt="Choose from the list" type="list">
       <formula1>"NONE,HOUSING,CREDIT,EMPLOYMENT,ISSUES_ELECTIONS_POLITICS,ONLINE_GAMBLING_AND_GAMING,FINANCIAL_PRODUCTS_SERVICES"</formula1>
     </dataValidation>
-    <dataValidation sqref="G2:G500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid value" error="Pick a valid bid_strategy" promptTitle="bid_strategy" prompt="Choose from the list" type="list">
+    <dataValidation sqref="G2:G500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid value" error="Pick a valid campaign_bid_strategy" promptTitle="campaign_bid_strategy" prompt="Choose from the list" type="list">
       <formula1>"LOWEST_COST_WITHOUT_CAP,LOWEST_COST_WITH_BID_CAP,COST_CAP,LOWEST_COST_WITH_MIN_ROAS"</formula1>
     </dataValidation>
-    <dataValidation sqref="I2:I500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid value" error="Pick a valid billing_event" promptTitle="billing_event" prompt="Choose from the list" type="list">
+    <dataValidation sqref="N2:N500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid value" error="Pick a valid bid_strategy" promptTitle="bid_strategy" prompt="Choose from the list" type="list">
+      <formula1>"LOWEST_COST_WITHOUT_CAP,LOWEST_COST_WITH_BID_CAP,COST_CAP,LOWEST_COST_WITH_MIN_ROAS"</formula1>
+    </dataValidation>
+    <dataValidation sqref="S2:S500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid value" error="Pick a valid pacing_type" promptTitle="pacing_type" prompt="Choose from the list" type="list">
+      <formula1>",standard,no_pacing"</formula1>
+    </dataValidation>
+    <dataValidation sqref="T2:T500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid value" error="Pick a valid billing_event" promptTitle="billing_event" prompt="Choose from the list" type="list">
       <formula1>"IMPRESSIONS,LINK_CLICKS,POST_ENGAGEMENT,VIDEO_VIEWS,THRUPLAY"</formula1>
     </dataValidation>
-    <dataValidation sqref="J2:J500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid value" error="Pick a valid optimization_goal" promptTitle="optimization_goal" prompt="Choose from the list" type="list">
+    <dataValidation sqref="U2:U500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid value" error="Pick a valid optimization_goal" promptTitle="optimization_goal" prompt="Choose from the list" type="list">
       <formula1>"REACH,IMPRESSIONS,LINK_CLICKS,LANDING_PAGE_VIEWS,POST_ENGAGEMENT,PAGE_LIKES,VIDEO_VIEWS,THRUPLAY,OFFSITE_CONVERSIONS,VALUE,LEAD_GENERATION,QUALITY_LEAD,CONVERSATIONS,APP_INSTALLS,AD_RECALL_LIFT"</formula1>
     </dataValidation>
-    <dataValidation sqref="K2:K500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid value" error="Pick a valid destination_type" promptTitle="destination_type" prompt="Choose from the list" type="list">
+    <dataValidation sqref="V2:V500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid value" error="Pick a valid destination_type" promptTitle="destination_type" prompt="Choose from the list" type="list">
       <formula1>"WEBSITE,APP,MESSENGER,INSTAGRAM_DIRECT,WHATSAPP,FACEBOOK,ON_AD,ON_POST,ON_PAGE,ON_EVENT,ON_VIDEO,SHOP_AUTOMATIC"</formula1>
     </dataValidation>
-    <dataValidation sqref="O2:O500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid value" error="Pick a valid custom_event_type" promptTitle="custom_event_type" prompt="Choose from the list" type="list">
+    <dataValidation sqref="Z2:Z500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid value" error="Pick a valid custom_event_type" promptTitle="custom_event_type" prompt="Choose from the list" type="list">
       <formula1>",PURCHASE,LEAD,COMPLETE_REGISTRATION,ADD_TO_CART,INITIATE_CHECKOUT,ADD_PAYMENT_INFO,VIEW_CONTENT,SEARCH,SUBSCRIBE,CONTACT,DONATE,OTHER"</formula1>
     </dataValidation>
-    <dataValidation sqref="AC2:AC500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid value" error="Pick a valid cta" promptTitle="cta" prompt="Choose from the list" type="list">
+    <dataValidation sqref="AI2:AI500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid value" error="Pick a valid genders" promptTitle="genders" prompt="Choose from the list" type="list">
+      <formula1>",1,2,1,2"</formula1>
+    </dataValidation>
+    <dataValidation sqref="AV2:AV500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid value" error="Pick a valid cta" promptTitle="cta" prompt="Choose from the list" type="list">
       <formula1>"SHOP_NOW,LEARN_MORE,SIGN_UP,SUBSCRIBE,DOWNLOAD,BOOK_TRAVEL,CONTACT_US,GET_OFFER,GET_QUOTE,APPLY_NOW,ORDER_NOW,DONATE_NOW,INSTALL_APP,USE_APP,WATCH_MORE,LISTEN_NOW,SEND_MESSAGE,MESSAGE_PAGE,GET_DIRECTIONS,CALL_NOW,NO_BUTTON"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
Add video_url column for one-step video uploads
Lets users paste a public video URL (Drive auto-converted) instead of
having to pre-upload the video to Meta's media library and find its
video_id. The script uploads via POST /act_<id>/advideos using
file_url, gets the video_id back, then builds the video creative as
usual. video_id and video_url are mutually exclusive.
</commit_message>
<xml_diff>
--- a/template.xlsx
+++ b/template.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:BC2"/>
+  <dimension ref="A1:BD2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -468,9 +468,10 @@
     <col width="14" customWidth="1" min="50" max="50"/>
     <col width="14" customWidth="1" min="51" max="51"/>
     <col width="14" customWidth="1" min="52" max="52"/>
-    <col width="15" customWidth="1" min="53" max="53"/>
-    <col width="14" customWidth="1" min="54" max="54"/>
-    <col width="19" customWidth="1" min="55" max="55"/>
+    <col width="14" customWidth="1" min="53" max="53"/>
+    <col width="15" customWidth="1" min="54" max="54"/>
+    <col width="14" customWidth="1" min="55" max="55"/>
+    <col width="19" customWidth="1" min="56" max="56"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -701,50 +702,55 @@
       </c>
       <c r="AT1" t="inlineStr">
         <is>
+          <t>video_url</t>
+        </is>
+      </c>
+      <c r="AU1" t="inlineStr">
+        <is>
           <t>primary_text</t>
         </is>
       </c>
-      <c r="AU1" t="inlineStr">
+      <c r="AV1" t="inlineStr">
         <is>
           <t>headline</t>
         </is>
       </c>
-      <c r="AV1" t="inlineStr">
+      <c r="AW1" t="inlineStr">
         <is>
           <t>description</t>
         </is>
       </c>
-      <c r="AW1" t="inlineStr">
+      <c r="AX1" t="inlineStr">
         <is>
           <t>link_url</t>
         </is>
       </c>
-      <c r="AX1" t="inlineStr">
+      <c r="AY1" t="inlineStr">
         <is>
           <t>display_link</t>
         </is>
       </c>
-      <c r="AY1" t="inlineStr">
+      <c r="AZ1" t="inlineStr">
         <is>
           <t>url_tags</t>
         </is>
       </c>
-      <c r="AZ1" t="inlineStr">
+      <c r="BA1" t="inlineStr">
         <is>
           <t>cta</t>
         </is>
       </c>
-      <c r="BA1" t="inlineStr">
+      <c r="BB1" t="inlineStr">
         <is>
           <t>browser_addon</t>
         </is>
       </c>
-      <c r="BB1" t="inlineStr">
+      <c r="BC1" t="inlineStr">
         <is>
           <t>phone_number</t>
         </is>
       </c>
-      <c r="BC1" t="inlineStr">
+      <c r="BD1" t="inlineStr">
         <is>
           <t>conversion_domain</t>
         </is>
@@ -854,44 +860,45 @@
         </is>
       </c>
       <c r="AS2" t="inlineStr"/>
-      <c r="AT2" t="inlineStr">
+      <c r="AT2" t="inlineStr"/>
+      <c r="AU2" t="inlineStr">
         <is>
           <t>Discover our new spring collection.</t>
         </is>
       </c>
-      <c r="AU2" t="inlineStr">
+      <c r="AV2" t="inlineStr">
         <is>
           <t>Spring is here</t>
         </is>
       </c>
-      <c r="AV2" t="inlineStr">
+      <c r="AW2" t="inlineStr">
         <is>
           <t>Shop the drop</t>
         </is>
       </c>
-      <c r="AW2" t="inlineStr">
+      <c r="AX2" t="inlineStr">
         <is>
           <t>https://example.com/spring</t>
         </is>
       </c>
-      <c r="AX2" t="inlineStr">
+      <c r="AY2" t="inlineStr">
         <is>
           <t>example.com</t>
         </is>
       </c>
-      <c r="AY2" t="inlineStr">
+      <c r="AZ2" t="inlineStr">
         <is>
           <t>utm_source=facebook&amp;utm_medium=cpc&amp;utm_campaign=spring</t>
         </is>
       </c>
-      <c r="AZ2" t="inlineStr">
+      <c r="BA2" t="inlineStr">
         <is>
           <t>SHOP_NOW</t>
         </is>
       </c>
-      <c r="BA2" t="inlineStr"/>
       <c r="BB2" t="inlineStr"/>
-      <c r="BC2" t="inlineStr">
+      <c r="BC2" t="inlineStr"/>
+      <c r="BD2" t="inlineStr">
         <is>
           <t>example.com</t>
         </is>
@@ -932,10 +939,10 @@
     <dataValidation sqref="AK2:AK500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid value" error="Pick a valid genders" promptTitle="genders" prompt="Choose from the list" type="list">
       <formula1>",1,2,1,2"</formula1>
     </dataValidation>
-    <dataValidation sqref="AZ2:AZ500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid value" error="Pick a valid cta" promptTitle="cta" prompt="Choose from the list" type="list">
+    <dataValidation sqref="BA2:BA500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid value" error="Pick a valid cta" promptTitle="cta" prompt="Choose from the list" type="list">
       <formula1>"SHOP_NOW,LEARN_MORE,SIGN_UP,SUBSCRIBE,DOWNLOAD,BOOK_TRAVEL,CONTACT_US,GET_OFFER,GET_QUOTE,APPLY_NOW,ORDER_NOW,DONATE_NOW,INSTALL_APP,USE_APP,WATCH_MORE,LISTEN_NOW,SEND_MESSAGE,MESSAGE_PAGE,GET_DIRECTIONS,CALL_NOW,NO_BUTTON"</formula1>
     </dataValidation>
-    <dataValidation sqref="BA2:BA500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid value" error="Pick a valid browser_addon" promptTitle="browser_addon" prompt="Choose from the list" type="list">
+    <dataValidation sqref="BB2:BB500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid value" error="Pick a valid browser_addon" promptTitle="browser_addon" prompt="Choose from the list" type="list">
       <formula1>",NONE,CALL,MESSENGER,WHATSAPP"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
Add columns for all visible Advantage+ creative features
Expands the per-feature column set from 7 to 14, covering every
toggle visible in Ads Manager's 'Advantage+ creative enhancements'
and 'Essential enhancements' sections:

  adv_add_overlays         -> ADD_TEXT_OVERLAY        (best-guess)
  adv_product_tags         -> PRODUCT_TAGS            (best-guess; catalog-only)
  adv_relevant_comments    -> RELEVANT_COMMENTS
  adv_enhance_cta          -> CTA_ENHANCEMENT
  adv_brightness_contrast  -> IMAGE_BRIGHTNESS_AND_CONTRAST
  adv_reveal_details       -> SHOWCASE_DESTINATION    (best-guess)
  adv_spotlights           -> CREATIVE_HIGHLIGHTING   (best-guess)

The four best-guess API keys may need adjustment based on Meta's
account-specific allowed list — error messages give the canonical
names.
</commit_message>
<xml_diff>
--- a/template.xlsx
+++ b/template.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:BL2"/>
+  <dimension ref="A1:BS2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -473,13 +473,20 @@
     <col width="14" customWidth="1" min="55" max="55"/>
     <col width="19" customWidth="1" min="56" max="56"/>
     <col width="25" customWidth="1" min="57" max="57"/>
-    <col width="21" customWidth="1" min="58" max="58"/>
+    <col width="18" customWidth="1" min="58" max="58"/>
     <col width="20" customWidth="1" min="59" max="59"/>
-    <col width="21" customWidth="1" min="60" max="60"/>
-    <col width="30" customWidth="1" min="61" max="61"/>
-    <col width="23" customWidth="1" min="62" max="62"/>
-    <col width="14" customWidth="1" min="63" max="63"/>
-    <col width="18" customWidth="1" min="64" max="64"/>
+    <col width="14" customWidth="1" min="60" max="60"/>
+    <col width="21" customWidth="1" min="61" max="61"/>
+    <col width="21" customWidth="1" min="62" max="62"/>
+    <col width="18" customWidth="1" min="63" max="63"/>
+    <col width="23" customWidth="1" min="64" max="64"/>
+    <col width="17" customWidth="1" min="65" max="65"/>
+    <col width="25" customWidth="1" min="66" max="66"/>
+    <col width="20" customWidth="1" min="67" max="67"/>
+    <col width="16" customWidth="1" min="68" max="68"/>
+    <col width="30" customWidth="1" min="69" max="69"/>
+    <col width="23" customWidth="1" min="70" max="70"/>
+    <col width="18" customWidth="1" min="71" max="71"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -770,35 +777,70 @@
       </c>
       <c r="BF1" t="inlineStr">
         <is>
+          <t>adv_add_overlays</t>
+        </is>
+      </c>
+      <c r="BG1" t="inlineStr">
+        <is>
+          <t>adv_image_touchups</t>
+        </is>
+      </c>
+      <c r="BH1" t="inlineStr">
+        <is>
+          <t>adv_music</t>
+        </is>
+      </c>
+      <c r="BI1" t="inlineStr">
+        <is>
+          <t>adv_text_generation</t>
+        </is>
+      </c>
+      <c r="BJ1" t="inlineStr">
+        <is>
           <t>adv_image_animation</t>
         </is>
       </c>
-      <c r="BG1" t="inlineStr">
-        <is>
-          <t>adv_image_touchups</t>
-        </is>
-      </c>
-      <c r="BH1" t="inlineStr">
-        <is>
-          <t>adv_text_generation</t>
-        </is>
-      </c>
-      <c r="BI1" t="inlineStr">
+      <c r="BK1" t="inlineStr">
+        <is>
+          <t>adv_product_tags</t>
+        </is>
+      </c>
+      <c r="BL1" t="inlineStr">
+        <is>
+          <t>adv_relevant_comments</t>
+        </is>
+      </c>
+      <c r="BM1" t="inlineStr">
+        <is>
+          <t>adv_enhance_cta</t>
+        </is>
+      </c>
+      <c r="BN1" t="inlineStr">
+        <is>
+          <t>adv_brightness_contrast</t>
+        </is>
+      </c>
+      <c r="BO1" t="inlineStr">
+        <is>
+          <t>adv_reveal_details</t>
+        </is>
+      </c>
+      <c r="BP1" t="inlineStr">
+        <is>
+          <t>adv_spotlights</t>
+        </is>
+      </c>
+      <c r="BQ1" t="inlineStr">
         <is>
           <t>adv_text_overlay_translation</t>
         </is>
       </c>
-      <c r="BJ1" t="inlineStr">
+      <c r="BR1" t="inlineStr">
         <is>
           <t>adv_ig_video_subtitle</t>
         </is>
       </c>
-      <c r="BK1" t="inlineStr">
-        <is>
-          <t>adv_music</t>
-        </is>
-      </c>
-      <c r="BL1" t="inlineStr">
+      <c r="BS1" t="inlineStr">
         <is>
           <t>adv_profile_card</t>
         </is>
@@ -959,9 +1001,16 @@
       <c r="BJ2" t="inlineStr"/>
       <c r="BK2" t="inlineStr"/>
       <c r="BL2" t="inlineStr"/>
+      <c r="BM2" t="inlineStr"/>
+      <c r="BN2" t="inlineStr"/>
+      <c r="BO2" t="inlineStr"/>
+      <c r="BP2" t="inlineStr"/>
+      <c r="BQ2" t="inlineStr"/>
+      <c r="BR2" t="inlineStr"/>
+      <c r="BS2" t="inlineStr"/>
     </row>
   </sheetData>
-  <dataValidations count="21">
+  <dataValidations count="28">
     <dataValidation sqref="C2:C500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid value" error="Pick a valid campaign_objective" promptTitle="campaign_objective" prompt="Choose from the list" type="list">
       <formula1>"OUTCOME_AWARENESS,OUTCOME_TRAFFIC,OUTCOME_ENGAGEMENT,OUTCOME_LEADS,OUTCOME_APP_PROMOTION,OUTCOME_SALES"</formula1>
     </dataValidation>
@@ -1004,25 +1053,46 @@
     <dataValidation sqref="BE2:BE500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid value" error="Pick a valid advantage_plus_creative" promptTitle="advantage_plus_creative" prompt="Choose from the list" type="list">
       <formula1>",ENABLED,DISABLED"</formula1>
     </dataValidation>
-    <dataValidation sqref="BF2:BF500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid value" error="Pick a valid adv_image_animation" promptTitle="adv_image_animation" prompt="Choose from the list" type="list">
+    <dataValidation sqref="BF2:BF500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid value" error="Pick a valid adv_add_overlays" promptTitle="adv_add_overlays" prompt="Choose from the list" type="list">
       <formula1>",OPT_IN,OPT_OUT"</formula1>
     </dataValidation>
     <dataValidation sqref="BG2:BG500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid value" error="Pick a valid adv_image_touchups" promptTitle="adv_image_touchups" prompt="Choose from the list" type="list">
       <formula1>",OPT_IN,OPT_OUT"</formula1>
     </dataValidation>
-    <dataValidation sqref="BH2:BH500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid value" error="Pick a valid adv_text_generation" promptTitle="adv_text_generation" prompt="Choose from the list" type="list">
-      <formula1>",OPT_IN,OPT_OUT"</formula1>
-    </dataValidation>
-    <dataValidation sqref="BI2:BI500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid value" error="Pick a valid adv_text_overlay_translation" promptTitle="adv_text_overlay_translation" prompt="Choose from the list" type="list">
-      <formula1>",OPT_IN,OPT_OUT"</formula1>
-    </dataValidation>
-    <dataValidation sqref="BJ2:BJ500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid value" error="Pick a valid adv_ig_video_subtitle" promptTitle="adv_ig_video_subtitle" prompt="Choose from the list" type="list">
-      <formula1>",OPT_IN,OPT_OUT"</formula1>
-    </dataValidation>
-    <dataValidation sqref="BK2:BK500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid value" error="Pick a valid adv_music" promptTitle="adv_music" prompt="Choose from the list" type="list">
-      <formula1>",OPT_IN,OPT_OUT"</formula1>
-    </dataValidation>
-    <dataValidation sqref="BL2:BL500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid value" error="Pick a valid adv_profile_card" promptTitle="adv_profile_card" prompt="Choose from the list" type="list">
+    <dataValidation sqref="BH2:BH500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid value" error="Pick a valid adv_music" promptTitle="adv_music" prompt="Choose from the list" type="list">
+      <formula1>",OPT_IN,OPT_OUT"</formula1>
+    </dataValidation>
+    <dataValidation sqref="BI2:BI500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid value" error="Pick a valid adv_text_generation" promptTitle="adv_text_generation" prompt="Choose from the list" type="list">
+      <formula1>",OPT_IN,OPT_OUT"</formula1>
+    </dataValidation>
+    <dataValidation sqref="BJ2:BJ500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid value" error="Pick a valid adv_image_animation" promptTitle="adv_image_animation" prompt="Choose from the list" type="list">
+      <formula1>",OPT_IN,OPT_OUT"</formula1>
+    </dataValidation>
+    <dataValidation sqref="BK2:BK500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid value" error="Pick a valid adv_product_tags" promptTitle="adv_product_tags" prompt="Choose from the list" type="list">
+      <formula1>",OPT_IN,OPT_OUT"</formula1>
+    </dataValidation>
+    <dataValidation sqref="BL2:BL500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid value" error="Pick a valid adv_relevant_comments" promptTitle="adv_relevant_comments" prompt="Choose from the list" type="list">
+      <formula1>",OPT_IN,OPT_OUT"</formula1>
+    </dataValidation>
+    <dataValidation sqref="BM2:BM500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid value" error="Pick a valid adv_enhance_cta" promptTitle="adv_enhance_cta" prompt="Choose from the list" type="list">
+      <formula1>",OPT_IN,OPT_OUT"</formula1>
+    </dataValidation>
+    <dataValidation sqref="BN2:BN500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid value" error="Pick a valid adv_brightness_contrast" promptTitle="adv_brightness_contrast" prompt="Choose from the list" type="list">
+      <formula1>",OPT_IN,OPT_OUT"</formula1>
+    </dataValidation>
+    <dataValidation sqref="BO2:BO500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid value" error="Pick a valid adv_reveal_details" promptTitle="adv_reveal_details" prompt="Choose from the list" type="list">
+      <formula1>",OPT_IN,OPT_OUT"</formula1>
+    </dataValidation>
+    <dataValidation sqref="BP2:BP500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid value" error="Pick a valid adv_spotlights" promptTitle="adv_spotlights" prompt="Choose from the list" type="list">
+      <formula1>",OPT_IN,OPT_OUT"</formula1>
+    </dataValidation>
+    <dataValidation sqref="BQ2:BQ500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid value" error="Pick a valid adv_text_overlay_translation" promptTitle="adv_text_overlay_translation" prompt="Choose from the list" type="list">
+      <formula1>",OPT_IN,OPT_OUT"</formula1>
+    </dataValidation>
+    <dataValidation sqref="BR2:BR500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid value" error="Pick a valid adv_ig_video_subtitle" promptTitle="adv_ig_video_subtitle" prompt="Choose from the list" type="list">
+      <formula1>",OPT_IN,OPT_OUT"</formula1>
+    </dataValidation>
+    <dataValidation sqref="BS2:BS500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid value" error="Pick a valid adv_profile_card" promptTitle="adv_profile_card" prompt="Choose from the list" type="list">
       <formula1>",OPT_IN,OPT_OUT"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
Add existing_post_id and partnership_ad_code columns
Both promote an existing Page post via the API's object_story_id
field (vs object_story_spec for new creatives):

  existing_post_id     -> your own Page's post. Accepts either a
                          bare POST_ID (combined with the row's
                          page_id) or the full PAGE_ID_POST_ID.
  partnership_ad_code  -> a Branded Content / Partnership Ad code
                          shared by a partner Page. Must be the
                          full PARTNER_PAGE_ID_POST_ID form because
                          the partner's Page ID is not the row's
                          page_id.

When either is set, all other creative-content columns (image_url,
headline, primary_text, link_url, cta, browser_addon, phone_number,
description, video_id, video_url, display_link) are ignored — the
existing post carries the content. Advantage+ features still apply.
</commit_message>
<xml_diff>
--- a/template.xlsx
+++ b/template.xlsx
@@ -443,7 +443,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:BS2"/>
+  <dimension ref="A1:BU2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -489,8 +489,8 @@
     <col width="19" customWidth="1" min="41" max="41"/>
     <col width="17" customWidth="1" min="42" max="42"/>
     <col width="14" customWidth="1" min="43" max="43"/>
-    <col width="14" customWidth="1" min="44" max="44"/>
-    <col width="14" customWidth="1" min="45" max="45"/>
+    <col width="18" customWidth="1" min="44" max="44"/>
+    <col width="21" customWidth="1" min="45" max="45"/>
     <col width="14" customWidth="1" min="46" max="46"/>
     <col width="14" customWidth="1" min="47" max="47"/>
     <col width="14" customWidth="1" min="48" max="48"/>
@@ -499,24 +499,26 @@
     <col width="14" customWidth="1" min="51" max="51"/>
     <col width="14" customWidth="1" min="52" max="52"/>
     <col width="14" customWidth="1" min="53" max="53"/>
-    <col width="15" customWidth="1" min="54" max="54"/>
+    <col width="14" customWidth="1" min="54" max="54"/>
     <col width="14" customWidth="1" min="55" max="55"/>
-    <col width="19" customWidth="1" min="56" max="56"/>
-    <col width="25" customWidth="1" min="57" max="57"/>
-    <col width="18" customWidth="1" min="58" max="58"/>
-    <col width="20" customWidth="1" min="59" max="59"/>
-    <col width="14" customWidth="1" min="60" max="60"/>
-    <col width="21" customWidth="1" min="61" max="61"/>
-    <col width="21" customWidth="1" min="62" max="62"/>
-    <col width="18" customWidth="1" min="63" max="63"/>
-    <col width="23" customWidth="1" min="64" max="64"/>
-    <col width="17" customWidth="1" min="65" max="65"/>
-    <col width="25" customWidth="1" min="66" max="66"/>
-    <col width="20" customWidth="1" min="67" max="67"/>
-    <col width="16" customWidth="1" min="68" max="68"/>
-    <col width="30" customWidth="1" min="69" max="69"/>
-    <col width="23" customWidth="1" min="70" max="70"/>
-    <col width="18" customWidth="1" min="71" max="71"/>
+    <col width="15" customWidth="1" min="56" max="56"/>
+    <col width="14" customWidth="1" min="57" max="57"/>
+    <col width="19" customWidth="1" min="58" max="58"/>
+    <col width="25" customWidth="1" min="59" max="59"/>
+    <col width="18" customWidth="1" min="60" max="60"/>
+    <col width="20" customWidth="1" min="61" max="61"/>
+    <col width="14" customWidth="1" min="62" max="62"/>
+    <col width="21" customWidth="1" min="63" max="63"/>
+    <col width="21" customWidth="1" min="64" max="64"/>
+    <col width="18" customWidth="1" min="65" max="65"/>
+    <col width="23" customWidth="1" min="66" max="66"/>
+    <col width="17" customWidth="1" min="67" max="67"/>
+    <col width="25" customWidth="1" min="68" max="68"/>
+    <col width="20" customWidth="1" min="69" max="69"/>
+    <col width="16" customWidth="1" min="70" max="70"/>
+    <col width="30" customWidth="1" min="71" max="71"/>
+    <col width="23" customWidth="1" min="72" max="72"/>
+    <col width="18" customWidth="1" min="73" max="73"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -737,140 +739,150 @@
       </c>
       <c r="AR1" t="inlineStr">
         <is>
+          <t>existing_post_id</t>
+        </is>
+      </c>
+      <c r="AS1" t="inlineStr">
+        <is>
+          <t>partnership_ad_code</t>
+        </is>
+      </c>
+      <c r="AT1" t="inlineStr">
+        <is>
           <t>image_url</t>
         </is>
       </c>
-      <c r="AS1" t="inlineStr">
+      <c r="AU1" t="inlineStr">
         <is>
           <t>video_id</t>
         </is>
       </c>
-      <c r="AT1" t="inlineStr">
+      <c r="AV1" t="inlineStr">
         <is>
           <t>video_url</t>
         </is>
       </c>
-      <c r="AU1" t="inlineStr">
+      <c r="AW1" t="inlineStr">
         <is>
           <t>primary_text</t>
         </is>
       </c>
-      <c r="AV1" t="inlineStr">
+      <c r="AX1" t="inlineStr">
         <is>
           <t>headline</t>
         </is>
       </c>
-      <c r="AW1" t="inlineStr">
+      <c r="AY1" t="inlineStr">
         <is>
           <t>description</t>
         </is>
       </c>
-      <c r="AX1" t="inlineStr">
+      <c r="AZ1" t="inlineStr">
         <is>
           <t>link_url</t>
         </is>
       </c>
-      <c r="AY1" t="inlineStr">
+      <c r="BA1" t="inlineStr">
         <is>
           <t>display_link</t>
         </is>
       </c>
-      <c r="AZ1" t="inlineStr">
+      <c r="BB1" t="inlineStr">
         <is>
           <t>url_tags</t>
         </is>
       </c>
-      <c r="BA1" t="inlineStr">
+      <c r="BC1" t="inlineStr">
         <is>
           <t>cta</t>
         </is>
       </c>
-      <c r="BB1" t="inlineStr">
+      <c r="BD1" t="inlineStr">
         <is>
           <t>browser_addon</t>
         </is>
       </c>
-      <c r="BC1" t="inlineStr">
+      <c r="BE1" t="inlineStr">
         <is>
           <t>phone_number</t>
         </is>
       </c>
-      <c r="BD1" t="inlineStr">
+      <c r="BF1" t="inlineStr">
         <is>
           <t>conversion_domain</t>
         </is>
       </c>
-      <c r="BE1" t="inlineStr">
+      <c r="BG1" t="inlineStr">
         <is>
           <t>advantage_plus_creative</t>
         </is>
       </c>
-      <c r="BF1" t="inlineStr">
+      <c r="BH1" t="inlineStr">
         <is>
           <t>adv_add_overlays</t>
         </is>
       </c>
-      <c r="BG1" t="inlineStr">
+      <c r="BI1" t="inlineStr">
         <is>
           <t>adv_image_touchups</t>
         </is>
       </c>
-      <c r="BH1" t="inlineStr">
+      <c r="BJ1" t="inlineStr">
         <is>
           <t>adv_music</t>
         </is>
       </c>
-      <c r="BI1" t="inlineStr">
+      <c r="BK1" t="inlineStr">
         <is>
           <t>adv_text_generation</t>
         </is>
       </c>
-      <c r="BJ1" t="inlineStr">
+      <c r="BL1" t="inlineStr">
         <is>
           <t>adv_image_animation</t>
         </is>
       </c>
-      <c r="BK1" t="inlineStr">
+      <c r="BM1" t="inlineStr">
         <is>
           <t>adv_product_tags</t>
         </is>
       </c>
-      <c r="BL1" t="inlineStr">
+      <c r="BN1" t="inlineStr">
         <is>
           <t>adv_relevant_comments</t>
         </is>
       </c>
-      <c r="BM1" t="inlineStr">
+      <c r="BO1" t="inlineStr">
         <is>
           <t>adv_enhance_cta</t>
         </is>
       </c>
-      <c r="BN1" t="inlineStr">
+      <c r="BP1" t="inlineStr">
         <is>
           <t>adv_brightness_contrast</t>
         </is>
       </c>
-      <c r="BO1" t="inlineStr">
+      <c r="BQ1" t="inlineStr">
         <is>
           <t>adv_reveal_details</t>
         </is>
       </c>
-      <c r="BP1" t="inlineStr">
+      <c r="BR1" t="inlineStr">
         <is>
           <t>adv_spotlights</t>
         </is>
       </c>
-      <c r="BQ1" t="inlineStr">
+      <c r="BS1" t="inlineStr">
         <is>
           <t>adv_text_overlay_translation</t>
         </is>
       </c>
-      <c r="BR1" t="inlineStr">
+      <c r="BT1" t="inlineStr">
         <is>
           <t>adv_ig_video_subtitle</t>
         </is>
       </c>
-      <c r="BS1" t="inlineStr">
+      <c r="BU1" t="inlineStr">
         <is>
           <t>adv_profile_card</t>
         </is>
@@ -974,53 +986,53 @@
           <t>My First Ad</t>
         </is>
       </c>
-      <c r="AR2" t="inlineStr">
+      <c r="AR2" t="inlineStr"/>
+      <c r="AS2" t="inlineStr"/>
+      <c r="AT2" t="inlineStr">
         <is>
           <t>https://example.com/image.jpg</t>
         </is>
       </c>
-      <c r="AS2" t="inlineStr"/>
-      <c r="AT2" t="inlineStr"/>
-      <c r="AU2" t="inlineStr">
+      <c r="AU2" t="inlineStr"/>
+      <c r="AV2" t="inlineStr"/>
+      <c r="AW2" t="inlineStr">
         <is>
           <t>Body copy goes here.</t>
         </is>
       </c>
-      <c r="AV2" t="inlineStr">
+      <c r="AX2" t="inlineStr">
         <is>
           <t>Your headline</t>
         </is>
       </c>
-      <c r="AW2" t="inlineStr">
+      <c r="AY2" t="inlineStr">
         <is>
           <t>Short description.</t>
         </is>
       </c>
-      <c r="AX2" t="inlineStr">
+      <c r="AZ2" t="inlineStr">
         <is>
           <t>https://example.com/landing</t>
         </is>
       </c>
-      <c r="AY2" t="inlineStr">
+      <c r="BA2" t="inlineStr">
         <is>
           <t>example.com</t>
         </is>
       </c>
-      <c r="AZ2" t="inlineStr"/>
-      <c r="BA2" t="inlineStr">
+      <c r="BB2" t="inlineStr"/>
+      <c r="BC2" t="inlineStr">
         <is>
           <t>SHOP_NOW</t>
         </is>
       </c>
-      <c r="BB2" t="inlineStr"/>
-      <c r="BC2" t="inlineStr"/>
-      <c r="BD2" t="inlineStr">
+      <c r="BD2" t="inlineStr"/>
+      <c r="BE2" t="inlineStr"/>
+      <c r="BF2" t="inlineStr">
         <is>
           <t>example.com</t>
         </is>
       </c>
-      <c r="BE2" t="inlineStr"/>
-      <c r="BF2" t="inlineStr"/>
       <c r="BG2" t="inlineStr"/>
       <c r="BH2" t="inlineStr"/>
       <c r="BI2" t="inlineStr"/>
@@ -1034,6 +1046,8 @@
       <c r="BQ2" t="inlineStr"/>
       <c r="BR2" t="inlineStr"/>
       <c r="BS2" t="inlineStr"/>
+      <c r="BT2" t="inlineStr"/>
+      <c r="BU2" t="inlineStr"/>
     </row>
   </sheetData>
   <dataValidations count="28">
@@ -1070,55 +1084,55 @@
     <dataValidation sqref="AK2:AK500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid value" error="Pick a valid genders" promptTitle="genders" prompt="Choose from the list" type="list">
       <formula1>genders_options</formula1>
     </dataValidation>
-    <dataValidation sqref="BA2:BA500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid value" error="Pick a valid cta" promptTitle="cta" prompt="Choose from the list" type="list">
+    <dataValidation sqref="BC2:BC500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid value" error="Pick a valid cta" promptTitle="cta" prompt="Choose from the list" type="list">
       <formula1>cta_options</formula1>
     </dataValidation>
-    <dataValidation sqref="BB2:BB500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid value" error="Pick a valid browser_addon" promptTitle="browser_addon" prompt="Choose from the list" type="list">
+    <dataValidation sqref="BD2:BD500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid value" error="Pick a valid browser_addon" promptTitle="browser_addon" prompt="Choose from the list" type="list">
       <formula1>browser_addon_options</formula1>
     </dataValidation>
-    <dataValidation sqref="BE2:BE500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid value" error="Pick a valid advantage_plus_creative" promptTitle="advantage_plus_creative" prompt="Choose from the list" type="list">
+    <dataValidation sqref="BG2:BG500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid value" error="Pick a valid advantage_plus_creative" promptTitle="advantage_plus_creative" prompt="Choose from the list" type="list">
       <formula1>advantage_plus_creative_options</formula1>
     </dataValidation>
-    <dataValidation sqref="BF2:BF500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid value" error="Pick a valid adv_add_overlays" promptTitle="adv_add_overlays" prompt="Choose from the list" type="list">
+    <dataValidation sqref="BH2:BH500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid value" error="Pick a valid adv_add_overlays" promptTitle="adv_add_overlays" prompt="Choose from the list" type="list">
       <formula1>adv_add_overlays_options</formula1>
     </dataValidation>
-    <dataValidation sqref="BG2:BG500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid value" error="Pick a valid adv_image_touchups" promptTitle="adv_image_touchups" prompt="Choose from the list" type="list">
+    <dataValidation sqref="BI2:BI500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid value" error="Pick a valid adv_image_touchups" promptTitle="adv_image_touchups" prompt="Choose from the list" type="list">
       <formula1>adv_image_touchups_options</formula1>
     </dataValidation>
-    <dataValidation sqref="BH2:BH500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid value" error="Pick a valid adv_music" promptTitle="adv_music" prompt="Choose from the list" type="list">
+    <dataValidation sqref="BJ2:BJ500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid value" error="Pick a valid adv_music" promptTitle="adv_music" prompt="Choose from the list" type="list">
       <formula1>adv_music_options</formula1>
     </dataValidation>
-    <dataValidation sqref="BI2:BI500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid value" error="Pick a valid adv_text_generation" promptTitle="adv_text_generation" prompt="Choose from the list" type="list">
+    <dataValidation sqref="BK2:BK500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid value" error="Pick a valid adv_text_generation" promptTitle="adv_text_generation" prompt="Choose from the list" type="list">
       <formula1>adv_text_generation_options</formula1>
     </dataValidation>
-    <dataValidation sqref="BJ2:BJ500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid value" error="Pick a valid adv_image_animation" promptTitle="adv_image_animation" prompt="Choose from the list" type="list">
+    <dataValidation sqref="BL2:BL500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid value" error="Pick a valid adv_image_animation" promptTitle="adv_image_animation" prompt="Choose from the list" type="list">
       <formula1>adv_image_animation_options</formula1>
     </dataValidation>
-    <dataValidation sqref="BK2:BK500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid value" error="Pick a valid adv_product_tags" promptTitle="adv_product_tags" prompt="Choose from the list" type="list">
+    <dataValidation sqref="BM2:BM500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid value" error="Pick a valid adv_product_tags" promptTitle="adv_product_tags" prompt="Choose from the list" type="list">
       <formula1>adv_product_tags_options</formula1>
     </dataValidation>
-    <dataValidation sqref="BL2:BL500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid value" error="Pick a valid adv_relevant_comments" promptTitle="adv_relevant_comments" prompt="Choose from the list" type="list">
+    <dataValidation sqref="BN2:BN500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid value" error="Pick a valid adv_relevant_comments" promptTitle="adv_relevant_comments" prompt="Choose from the list" type="list">
       <formula1>adv_relevant_comments_options</formula1>
     </dataValidation>
-    <dataValidation sqref="BM2:BM500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid value" error="Pick a valid adv_enhance_cta" promptTitle="adv_enhance_cta" prompt="Choose from the list" type="list">
+    <dataValidation sqref="BO2:BO500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid value" error="Pick a valid adv_enhance_cta" promptTitle="adv_enhance_cta" prompt="Choose from the list" type="list">
       <formula1>adv_enhance_cta_options</formula1>
     </dataValidation>
-    <dataValidation sqref="BN2:BN500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid value" error="Pick a valid adv_brightness_contrast" promptTitle="adv_brightness_contrast" prompt="Choose from the list" type="list">
+    <dataValidation sqref="BP2:BP500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid value" error="Pick a valid adv_brightness_contrast" promptTitle="adv_brightness_contrast" prompt="Choose from the list" type="list">
       <formula1>adv_brightness_contrast_options</formula1>
     </dataValidation>
-    <dataValidation sqref="BO2:BO500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid value" error="Pick a valid adv_reveal_details" promptTitle="adv_reveal_details" prompt="Choose from the list" type="list">
+    <dataValidation sqref="BQ2:BQ500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid value" error="Pick a valid adv_reveal_details" promptTitle="adv_reveal_details" prompt="Choose from the list" type="list">
       <formula1>adv_reveal_details_options</formula1>
     </dataValidation>
-    <dataValidation sqref="BP2:BP500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid value" error="Pick a valid adv_spotlights" promptTitle="adv_spotlights" prompt="Choose from the list" type="list">
+    <dataValidation sqref="BR2:BR500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid value" error="Pick a valid adv_spotlights" promptTitle="adv_spotlights" prompt="Choose from the list" type="list">
       <formula1>adv_spotlights_options</formula1>
     </dataValidation>
-    <dataValidation sqref="BQ2:BQ500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid value" error="Pick a valid adv_text_overlay_translation" promptTitle="adv_text_overlay_translation" prompt="Choose from the list" type="list">
+    <dataValidation sqref="BS2:BS500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid value" error="Pick a valid adv_text_overlay_translation" promptTitle="adv_text_overlay_translation" prompt="Choose from the list" type="list">
       <formula1>adv_text_overlay_translation_options</formula1>
     </dataValidation>
-    <dataValidation sqref="BR2:BR500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid value" error="Pick a valid adv_ig_video_subtitle" promptTitle="adv_ig_video_subtitle" prompt="Choose from the list" type="list">
+    <dataValidation sqref="BT2:BT500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid value" error="Pick a valid adv_ig_video_subtitle" promptTitle="adv_ig_video_subtitle" prompt="Choose from the list" type="list">
       <formula1>adv_ig_video_subtitle_options</formula1>
     </dataValidation>
-    <dataValidation sqref="BS2:BS500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid value" error="Pick a valid adv_profile_card" promptTitle="adv_profile_card" prompt="Choose from the list" type="list">
+    <dataValidation sqref="BU2:BU500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid value" error="Pick a valid adv_profile_card" promptTitle="adv_profile_card" prompt="Choose from the list" type="list">
       <formula1>adv_profile_card_options</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
Replace sponsor_*_id columns with Ads Manager's Second identity model
Ads Manager exposes partnership identity as 'Second identity' (Page
+ IG) plus a radio for 'Identities to display in the header'. New
columns mirror that:

  second_identity_page_id  -> sponsor FB Page  (was branded_content_sponsor_page_id)
  second_identity_ig_id    -> sponsor IG       (was branded_content_sponsor_ig_id)
  identity_display         -> DYNAMIC / BOTH / FIRST_ONLY

API mapping:
  second_identity_page_id  -> branded_content_sharing_partner_id
  second_identity_ig_id    -> instagram_user_id (creative-level override)
  identity_display         -> branded_content_identity_display (best-guess)

Defaults: when blank, second_identity_page_id falls back to the row's
page_id and second_identity_ig_id falls back to instagram_user_id.
</commit_message>
<xml_diff>
--- a/template.xlsx
+++ b/template.xlsx
@@ -22,23 +22,24 @@
     <definedName name="destination_type_options">'_options'!$I$2:$I$13</definedName>
     <definedName name="custom_event_type_options">'_options'!$J$2:$J$13</definedName>
     <definedName name="genders_options">'_options'!$K$2:$K$4</definedName>
-    <definedName name="cta_options">'_options'!$L$2:$L$22</definedName>
-    <definedName name="browser_addon_options">'_options'!$M$2:$M$5</definedName>
-    <definedName name="advantage_plus_creative_options">'_options'!$N$2:$N$3</definedName>
-    <definedName name="adv_add_overlays_options">'_options'!$O$2:$O$3</definedName>
-    <definedName name="adv_image_touchups_options">'_options'!$P$2:$P$3</definedName>
-    <definedName name="adv_music_options">'_options'!$Q$2:$Q$3</definedName>
-    <definedName name="adv_text_generation_options">'_options'!$R$2:$R$3</definedName>
-    <definedName name="adv_image_animation_options">'_options'!$S$2:$S$3</definedName>
-    <definedName name="adv_product_tags_options">'_options'!$T$2:$T$3</definedName>
-    <definedName name="adv_relevant_comments_options">'_options'!$U$2:$U$3</definedName>
-    <definedName name="adv_enhance_cta_options">'_options'!$V$2:$V$3</definedName>
-    <definedName name="adv_brightness_contrast_options">'_options'!$W$2:$W$3</definedName>
-    <definedName name="adv_reveal_details_options">'_options'!$X$2:$X$3</definedName>
-    <definedName name="adv_spotlights_options">'_options'!$Y$2:$Y$3</definedName>
-    <definedName name="adv_text_overlay_translation_options">'_options'!$Z$2:$Z$3</definedName>
-    <definedName name="adv_ig_video_subtitle_options">'_options'!$AA$2:$AA$3</definedName>
-    <definedName name="adv_profile_card_options">'_options'!$AB$2:$AB$3</definedName>
+    <definedName name="identity_display_options">'_options'!$L$2:$L$4</definedName>
+    <definedName name="cta_options">'_options'!$M$2:$M$22</definedName>
+    <definedName name="browser_addon_options">'_options'!$N$2:$N$5</definedName>
+    <definedName name="advantage_plus_creative_options">'_options'!$O$2:$O$3</definedName>
+    <definedName name="adv_add_overlays_options">'_options'!$P$2:$P$3</definedName>
+    <definedName name="adv_image_touchups_options">'_options'!$Q$2:$Q$3</definedName>
+    <definedName name="adv_music_options">'_options'!$R$2:$R$3</definedName>
+    <definedName name="adv_text_generation_options">'_options'!$S$2:$S$3</definedName>
+    <definedName name="adv_image_animation_options">'_options'!$T$2:$T$3</definedName>
+    <definedName name="adv_product_tags_options">'_options'!$U$2:$U$3</definedName>
+    <definedName name="adv_relevant_comments_options">'_options'!$V$2:$V$3</definedName>
+    <definedName name="adv_enhance_cta_options">'_options'!$W$2:$W$3</definedName>
+    <definedName name="adv_brightness_contrast_options">'_options'!$X$2:$X$3</definedName>
+    <definedName name="adv_reveal_details_options">'_options'!$Y$2:$Y$3</definedName>
+    <definedName name="adv_spotlights_options">'_options'!$Z$2:$Z$3</definedName>
+    <definedName name="adv_text_overlay_translation_options">'_options'!$AA$2:$AA$3</definedName>
+    <definedName name="adv_ig_video_subtitle_options">'_options'!$AB$2:$AB$3</definedName>
+    <definedName name="adv_profile_card_options">'_options'!$AC$2:$AC$3</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -443,7 +444,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:BW2"/>
+  <dimension ref="A1:BX2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -491,9 +492,9 @@
     <col width="14" customWidth="1" min="43" max="43"/>
     <col width="18" customWidth="1" min="44" max="44"/>
     <col width="21" customWidth="1" min="45" max="45"/>
-    <col width="33" customWidth="1" min="46" max="46"/>
-    <col width="31" customWidth="1" min="47" max="47"/>
-    <col width="14" customWidth="1" min="48" max="48"/>
+    <col width="25" customWidth="1" min="46" max="46"/>
+    <col width="23" customWidth="1" min="47" max="47"/>
+    <col width="18" customWidth="1" min="48" max="48"/>
     <col width="14" customWidth="1" min="49" max="49"/>
     <col width="14" customWidth="1" min="50" max="50"/>
     <col width="14" customWidth="1" min="51" max="51"/>
@@ -503,24 +504,25 @@
     <col width="14" customWidth="1" min="55" max="55"/>
     <col width="14" customWidth="1" min="56" max="56"/>
     <col width="14" customWidth="1" min="57" max="57"/>
-    <col width="15" customWidth="1" min="58" max="58"/>
-    <col width="14" customWidth="1" min="59" max="59"/>
-    <col width="19" customWidth="1" min="60" max="60"/>
-    <col width="25" customWidth="1" min="61" max="61"/>
-    <col width="18" customWidth="1" min="62" max="62"/>
-    <col width="20" customWidth="1" min="63" max="63"/>
-    <col width="14" customWidth="1" min="64" max="64"/>
-    <col width="21" customWidth="1" min="65" max="65"/>
+    <col width="14" customWidth="1" min="58" max="58"/>
+    <col width="15" customWidth="1" min="59" max="59"/>
+    <col width="14" customWidth="1" min="60" max="60"/>
+    <col width="19" customWidth="1" min="61" max="61"/>
+    <col width="25" customWidth="1" min="62" max="62"/>
+    <col width="18" customWidth="1" min="63" max="63"/>
+    <col width="20" customWidth="1" min="64" max="64"/>
+    <col width="14" customWidth="1" min="65" max="65"/>
     <col width="21" customWidth="1" min="66" max="66"/>
-    <col width="18" customWidth="1" min="67" max="67"/>
-    <col width="23" customWidth="1" min="68" max="68"/>
-    <col width="17" customWidth="1" min="69" max="69"/>
-    <col width="25" customWidth="1" min="70" max="70"/>
-    <col width="20" customWidth="1" min="71" max="71"/>
-    <col width="16" customWidth="1" min="72" max="72"/>
-    <col width="30" customWidth="1" min="73" max="73"/>
-    <col width="23" customWidth="1" min="74" max="74"/>
-    <col width="18" customWidth="1" min="75" max="75"/>
+    <col width="21" customWidth="1" min="67" max="67"/>
+    <col width="18" customWidth="1" min="68" max="68"/>
+    <col width="23" customWidth="1" min="69" max="69"/>
+    <col width="17" customWidth="1" min="70" max="70"/>
+    <col width="25" customWidth="1" min="71" max="71"/>
+    <col width="20" customWidth="1" min="72" max="72"/>
+    <col width="16" customWidth="1" min="73" max="73"/>
+    <col width="30" customWidth="1" min="74" max="74"/>
+    <col width="23" customWidth="1" min="75" max="75"/>
+    <col width="18" customWidth="1" min="76" max="76"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -751,150 +753,155 @@
       </c>
       <c r="AT1" t="inlineStr">
         <is>
-          <t>branded_content_sponsor_page_id</t>
+          <t>second_identity_page_id</t>
         </is>
       </c>
       <c r="AU1" t="inlineStr">
         <is>
-          <t>branded_content_sponsor_ig_id</t>
+          <t>second_identity_ig_id</t>
         </is>
       </c>
       <c r="AV1" t="inlineStr">
         <is>
+          <t>identity_display</t>
+        </is>
+      </c>
+      <c r="AW1" t="inlineStr">
+        <is>
           <t>image_url</t>
         </is>
       </c>
-      <c r="AW1" t="inlineStr">
+      <c r="AX1" t="inlineStr">
         <is>
           <t>video_id</t>
         </is>
       </c>
-      <c r="AX1" t="inlineStr">
+      <c r="AY1" t="inlineStr">
         <is>
           <t>video_url</t>
         </is>
       </c>
-      <c r="AY1" t="inlineStr">
+      <c r="AZ1" t="inlineStr">
         <is>
           <t>primary_text</t>
         </is>
       </c>
-      <c r="AZ1" t="inlineStr">
+      <c r="BA1" t="inlineStr">
         <is>
           <t>headline</t>
         </is>
       </c>
-      <c r="BA1" t="inlineStr">
+      <c r="BB1" t="inlineStr">
         <is>
           <t>description</t>
         </is>
       </c>
-      <c r="BB1" t="inlineStr">
+      <c r="BC1" t="inlineStr">
         <is>
           <t>link_url</t>
         </is>
       </c>
-      <c r="BC1" t="inlineStr">
+      <c r="BD1" t="inlineStr">
         <is>
           <t>display_link</t>
         </is>
       </c>
-      <c r="BD1" t="inlineStr">
+      <c r="BE1" t="inlineStr">
         <is>
           <t>url_tags</t>
         </is>
       </c>
-      <c r="BE1" t="inlineStr">
+      <c r="BF1" t="inlineStr">
         <is>
           <t>cta</t>
         </is>
       </c>
-      <c r="BF1" t="inlineStr">
+      <c r="BG1" t="inlineStr">
         <is>
           <t>browser_addon</t>
         </is>
       </c>
-      <c r="BG1" t="inlineStr">
+      <c r="BH1" t="inlineStr">
         <is>
           <t>phone_number</t>
         </is>
       </c>
-      <c r="BH1" t="inlineStr">
+      <c r="BI1" t="inlineStr">
         <is>
           <t>conversion_domain</t>
         </is>
       </c>
-      <c r="BI1" t="inlineStr">
+      <c r="BJ1" t="inlineStr">
         <is>
           <t>advantage_plus_creative</t>
         </is>
       </c>
-      <c r="BJ1" t="inlineStr">
+      <c r="BK1" t="inlineStr">
         <is>
           <t>adv_add_overlays</t>
         </is>
       </c>
-      <c r="BK1" t="inlineStr">
+      <c r="BL1" t="inlineStr">
         <is>
           <t>adv_image_touchups</t>
         </is>
       </c>
-      <c r="BL1" t="inlineStr">
+      <c r="BM1" t="inlineStr">
         <is>
           <t>adv_music</t>
         </is>
       </c>
-      <c r="BM1" t="inlineStr">
+      <c r="BN1" t="inlineStr">
         <is>
           <t>adv_text_generation</t>
         </is>
       </c>
-      <c r="BN1" t="inlineStr">
+      <c r="BO1" t="inlineStr">
         <is>
           <t>adv_image_animation</t>
         </is>
       </c>
-      <c r="BO1" t="inlineStr">
+      <c r="BP1" t="inlineStr">
         <is>
           <t>adv_product_tags</t>
         </is>
       </c>
-      <c r="BP1" t="inlineStr">
+      <c r="BQ1" t="inlineStr">
         <is>
           <t>adv_relevant_comments</t>
         </is>
       </c>
-      <c r="BQ1" t="inlineStr">
+      <c r="BR1" t="inlineStr">
         <is>
           <t>adv_enhance_cta</t>
         </is>
       </c>
-      <c r="BR1" t="inlineStr">
+      <c r="BS1" t="inlineStr">
         <is>
           <t>adv_brightness_contrast</t>
         </is>
       </c>
-      <c r="BS1" t="inlineStr">
+      <c r="BT1" t="inlineStr">
         <is>
           <t>adv_reveal_details</t>
         </is>
       </c>
-      <c r="BT1" t="inlineStr">
+      <c r="BU1" t="inlineStr">
         <is>
           <t>adv_spotlights</t>
         </is>
       </c>
-      <c r="BU1" t="inlineStr">
+      <c r="BV1" t="inlineStr">
         <is>
           <t>adv_text_overlay_translation</t>
         </is>
       </c>
-      <c r="BV1" t="inlineStr">
+      <c r="BW1" t="inlineStr">
         <is>
           <t>adv_ig_video_subtitle</t>
         </is>
       </c>
-      <c r="BW1" t="inlineStr">
+      <c r="BX1" t="inlineStr">
         <is>
           <t>adv_profile_card</t>
         </is>
@@ -1002,52 +1009,52 @@
       <c r="AS2" t="inlineStr"/>
       <c r="AT2" t="inlineStr"/>
       <c r="AU2" t="inlineStr"/>
-      <c r="AV2" t="inlineStr">
+      <c r="AV2" t="inlineStr"/>
+      <c r="AW2" t="inlineStr">
         <is>
           <t>https://example.com/image.jpg</t>
         </is>
       </c>
-      <c r="AW2" t="inlineStr"/>
       <c r="AX2" t="inlineStr"/>
-      <c r="AY2" t="inlineStr">
+      <c r="AY2" t="inlineStr"/>
+      <c r="AZ2" t="inlineStr">
         <is>
           <t>Body copy goes here.</t>
         </is>
       </c>
-      <c r="AZ2" t="inlineStr">
+      <c r="BA2" t="inlineStr">
         <is>
           <t>Your headline</t>
         </is>
       </c>
-      <c r="BA2" t="inlineStr">
+      <c r="BB2" t="inlineStr">
         <is>
           <t>Short description.</t>
         </is>
       </c>
-      <c r="BB2" t="inlineStr">
+      <c r="BC2" t="inlineStr">
         <is>
           <t>https://example.com/landing</t>
         </is>
       </c>
-      <c r="BC2" t="inlineStr">
+      <c r="BD2" t="inlineStr">
         <is>
           <t>example.com</t>
         </is>
       </c>
-      <c r="BD2" t="inlineStr"/>
-      <c r="BE2" t="inlineStr">
+      <c r="BE2" t="inlineStr"/>
+      <c r="BF2" t="inlineStr">
         <is>
           <t>SHOP_NOW</t>
         </is>
       </c>
-      <c r="BF2" t="inlineStr"/>
       <c r="BG2" t="inlineStr"/>
-      <c r="BH2" t="inlineStr">
+      <c r="BH2" t="inlineStr"/>
+      <c r="BI2" t="inlineStr">
         <is>
           <t>example.com</t>
         </is>
       </c>
-      <c r="BI2" t="inlineStr"/>
       <c r="BJ2" t="inlineStr"/>
       <c r="BK2" t="inlineStr"/>
       <c r="BL2" t="inlineStr"/>
@@ -1062,9 +1069,10 @@
       <c r="BU2" t="inlineStr"/>
       <c r="BV2" t="inlineStr"/>
       <c r="BW2" t="inlineStr"/>
+      <c r="BX2" t="inlineStr"/>
     </row>
   </sheetData>
-  <dataValidations count="28">
+  <dataValidations count="29">
     <dataValidation sqref="C2:C500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid value" error="Pick a valid campaign_objective" promptTitle="campaign_objective" prompt="Choose from the list" type="list">
       <formula1>campaign_objective_options</formula1>
     </dataValidation>
@@ -1098,55 +1106,58 @@
     <dataValidation sqref="AK2:AK500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid value" error="Pick a valid genders" promptTitle="genders" prompt="Choose from the list" type="list">
       <formula1>genders_options</formula1>
     </dataValidation>
-    <dataValidation sqref="BE2:BE500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid value" error="Pick a valid cta" promptTitle="cta" prompt="Choose from the list" type="list">
+    <dataValidation sqref="AV2:AV500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid value" error="Pick a valid identity_display" promptTitle="identity_display" prompt="Choose from the list" type="list">
+      <formula1>identity_display_options</formula1>
+    </dataValidation>
+    <dataValidation sqref="BF2:BF500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid value" error="Pick a valid cta" promptTitle="cta" prompt="Choose from the list" type="list">
       <formula1>cta_options</formula1>
     </dataValidation>
-    <dataValidation sqref="BF2:BF500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid value" error="Pick a valid browser_addon" promptTitle="browser_addon" prompt="Choose from the list" type="list">
+    <dataValidation sqref="BG2:BG500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid value" error="Pick a valid browser_addon" promptTitle="browser_addon" prompt="Choose from the list" type="list">
       <formula1>browser_addon_options</formula1>
     </dataValidation>
-    <dataValidation sqref="BI2:BI500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid value" error="Pick a valid advantage_plus_creative" promptTitle="advantage_plus_creative" prompt="Choose from the list" type="list">
+    <dataValidation sqref="BJ2:BJ500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid value" error="Pick a valid advantage_plus_creative" promptTitle="advantage_plus_creative" prompt="Choose from the list" type="list">
       <formula1>advantage_plus_creative_options</formula1>
     </dataValidation>
-    <dataValidation sqref="BJ2:BJ500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid value" error="Pick a valid adv_add_overlays" promptTitle="adv_add_overlays" prompt="Choose from the list" type="list">
+    <dataValidation sqref="BK2:BK500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid value" error="Pick a valid adv_add_overlays" promptTitle="adv_add_overlays" prompt="Choose from the list" type="list">
       <formula1>adv_add_overlays_options</formula1>
     </dataValidation>
-    <dataValidation sqref="BK2:BK500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid value" error="Pick a valid adv_image_touchups" promptTitle="adv_image_touchups" prompt="Choose from the list" type="list">
+    <dataValidation sqref="BL2:BL500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid value" error="Pick a valid adv_image_touchups" promptTitle="adv_image_touchups" prompt="Choose from the list" type="list">
       <formula1>adv_image_touchups_options</formula1>
     </dataValidation>
-    <dataValidation sqref="BL2:BL500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid value" error="Pick a valid adv_music" promptTitle="adv_music" prompt="Choose from the list" type="list">
+    <dataValidation sqref="BM2:BM500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid value" error="Pick a valid adv_music" promptTitle="adv_music" prompt="Choose from the list" type="list">
       <formula1>adv_music_options</formula1>
     </dataValidation>
-    <dataValidation sqref="BM2:BM500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid value" error="Pick a valid adv_text_generation" promptTitle="adv_text_generation" prompt="Choose from the list" type="list">
+    <dataValidation sqref="BN2:BN500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid value" error="Pick a valid adv_text_generation" promptTitle="adv_text_generation" prompt="Choose from the list" type="list">
       <formula1>adv_text_generation_options</formula1>
     </dataValidation>
-    <dataValidation sqref="BN2:BN500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid value" error="Pick a valid adv_image_animation" promptTitle="adv_image_animation" prompt="Choose from the list" type="list">
+    <dataValidation sqref="BO2:BO500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid value" error="Pick a valid adv_image_animation" promptTitle="adv_image_animation" prompt="Choose from the list" type="list">
       <formula1>adv_image_animation_options</formula1>
     </dataValidation>
-    <dataValidation sqref="BO2:BO500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid value" error="Pick a valid adv_product_tags" promptTitle="adv_product_tags" prompt="Choose from the list" type="list">
+    <dataValidation sqref="BP2:BP500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid value" error="Pick a valid adv_product_tags" promptTitle="adv_product_tags" prompt="Choose from the list" type="list">
       <formula1>adv_product_tags_options</formula1>
     </dataValidation>
-    <dataValidation sqref="BP2:BP500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid value" error="Pick a valid adv_relevant_comments" promptTitle="adv_relevant_comments" prompt="Choose from the list" type="list">
+    <dataValidation sqref="BQ2:BQ500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid value" error="Pick a valid adv_relevant_comments" promptTitle="adv_relevant_comments" prompt="Choose from the list" type="list">
       <formula1>adv_relevant_comments_options</formula1>
     </dataValidation>
-    <dataValidation sqref="BQ2:BQ500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid value" error="Pick a valid adv_enhance_cta" promptTitle="adv_enhance_cta" prompt="Choose from the list" type="list">
+    <dataValidation sqref="BR2:BR500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid value" error="Pick a valid adv_enhance_cta" promptTitle="adv_enhance_cta" prompt="Choose from the list" type="list">
       <formula1>adv_enhance_cta_options</formula1>
     </dataValidation>
-    <dataValidation sqref="BR2:BR500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid value" error="Pick a valid adv_brightness_contrast" promptTitle="adv_brightness_contrast" prompt="Choose from the list" type="list">
+    <dataValidation sqref="BS2:BS500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid value" error="Pick a valid adv_brightness_contrast" promptTitle="adv_brightness_contrast" prompt="Choose from the list" type="list">
       <formula1>adv_brightness_contrast_options</formula1>
     </dataValidation>
-    <dataValidation sqref="BS2:BS500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid value" error="Pick a valid adv_reveal_details" promptTitle="adv_reveal_details" prompt="Choose from the list" type="list">
+    <dataValidation sqref="BT2:BT500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid value" error="Pick a valid adv_reveal_details" promptTitle="adv_reveal_details" prompt="Choose from the list" type="list">
       <formula1>adv_reveal_details_options</formula1>
     </dataValidation>
-    <dataValidation sqref="BT2:BT500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid value" error="Pick a valid adv_spotlights" promptTitle="adv_spotlights" prompt="Choose from the list" type="list">
+    <dataValidation sqref="BU2:BU500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid value" error="Pick a valid adv_spotlights" promptTitle="adv_spotlights" prompt="Choose from the list" type="list">
       <formula1>adv_spotlights_options</formula1>
     </dataValidation>
-    <dataValidation sqref="BU2:BU500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid value" error="Pick a valid adv_text_overlay_translation" promptTitle="adv_text_overlay_translation" prompt="Choose from the list" type="list">
+    <dataValidation sqref="BV2:BV500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid value" error="Pick a valid adv_text_overlay_translation" promptTitle="adv_text_overlay_translation" prompt="Choose from the list" type="list">
       <formula1>adv_text_overlay_translation_options</formula1>
     </dataValidation>
-    <dataValidation sqref="BV2:BV500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid value" error="Pick a valid adv_ig_video_subtitle" promptTitle="adv_ig_video_subtitle" prompt="Choose from the list" type="list">
+    <dataValidation sqref="BW2:BW500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid value" error="Pick a valid adv_ig_video_subtitle" promptTitle="adv_ig_video_subtitle" prompt="Choose from the list" type="list">
       <formula1>adv_ig_video_subtitle_options</formula1>
     </dataValidation>
-    <dataValidation sqref="BW2:BW500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid value" error="Pick a valid adv_profile_card" promptTitle="adv_profile_card" prompt="Choose from the list" type="list">
+    <dataValidation sqref="BX2:BX500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid value" error="Pick a valid adv_profile_card" promptTitle="adv_profile_card" prompt="Choose from the list" type="list">
       <formula1>adv_profile_card_options</formula1>
     </dataValidation>
   </dataValidations>
@@ -1160,7 +1171,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AB22"/>
+  <dimension ref="A1:AC22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1221,85 +1232,90 @@
       </c>
       <c r="L1" t="inlineStr">
         <is>
+          <t>identity_display</t>
+        </is>
+      </c>
+      <c r="M1" t="inlineStr">
+        <is>
           <t>cta</t>
         </is>
       </c>
-      <c r="M1" t="inlineStr">
+      <c r="N1" t="inlineStr">
         <is>
           <t>browser_addon</t>
         </is>
       </c>
-      <c r="N1" t="inlineStr">
+      <c r="O1" t="inlineStr">
         <is>
           <t>advantage_plus_creative</t>
         </is>
       </c>
-      <c r="O1" t="inlineStr">
+      <c r="P1" t="inlineStr">
         <is>
           <t>adv_add_overlays</t>
         </is>
       </c>
-      <c r="P1" t="inlineStr">
+      <c r="Q1" t="inlineStr">
         <is>
           <t>adv_image_touchups</t>
         </is>
       </c>
-      <c r="Q1" t="inlineStr">
+      <c r="R1" t="inlineStr">
         <is>
           <t>adv_music</t>
         </is>
       </c>
-      <c r="R1" t="inlineStr">
+      <c r="S1" t="inlineStr">
         <is>
           <t>adv_text_generation</t>
         </is>
       </c>
-      <c r="S1" t="inlineStr">
+      <c r="T1" t="inlineStr">
         <is>
           <t>adv_image_animation</t>
         </is>
       </c>
-      <c r="T1" t="inlineStr">
+      <c r="U1" t="inlineStr">
         <is>
           <t>adv_product_tags</t>
         </is>
       </c>
-      <c r="U1" t="inlineStr">
+      <c r="V1" t="inlineStr">
         <is>
           <t>adv_relevant_comments</t>
         </is>
       </c>
-      <c r="V1" t="inlineStr">
+      <c r="W1" t="inlineStr">
         <is>
           <t>adv_enhance_cta</t>
         </is>
       </c>
-      <c r="W1" t="inlineStr">
+      <c r="X1" t="inlineStr">
         <is>
           <t>adv_brightness_contrast</t>
         </is>
       </c>
-      <c r="X1" t="inlineStr">
+      <c r="Y1" t="inlineStr">
         <is>
           <t>adv_reveal_details</t>
         </is>
       </c>
-      <c r="Y1" t="inlineStr">
+      <c r="Z1" t="inlineStr">
         <is>
           <t>adv_spotlights</t>
         </is>
       </c>
-      <c r="Z1" t="inlineStr">
+      <c r="AA1" t="inlineStr">
         <is>
           <t>adv_text_overlay_translation</t>
         </is>
       </c>
-      <c r="AA1" t="inlineStr">
+      <c r="AB1" t="inlineStr">
         <is>
           <t>adv_ig_video_subtitle</t>
         </is>
       </c>
-      <c r="AB1" t="inlineStr">
+      <c r="AC1" t="inlineStr">
         <is>
           <t>adv_profile_card</t>
         </is>
@@ -1363,85 +1379,90 @@
       </c>
       <c r="L2" t="inlineStr">
         <is>
+          <t>DYNAMIC</t>
+        </is>
+      </c>
+      <c r="M2" t="inlineStr">
+        <is>
           <t>SHOP_NOW</t>
         </is>
       </c>
-      <c r="M2" t="inlineStr">
+      <c r="N2" t="inlineStr">
         <is>
           <t>NONE</t>
         </is>
       </c>
-      <c r="N2" t="inlineStr">
+      <c r="O2" t="inlineStr">
         <is>
           <t>ON</t>
         </is>
       </c>
-      <c r="O2" t="inlineStr">
+      <c r="P2" t="inlineStr">
         <is>
           <t>ON</t>
         </is>
       </c>
-      <c r="P2" t="inlineStr">
+      <c r="Q2" t="inlineStr">
         <is>
           <t>ON</t>
         </is>
       </c>
-      <c r="Q2" t="inlineStr">
+      <c r="R2" t="inlineStr">
         <is>
           <t>ON</t>
         </is>
       </c>
-      <c r="R2" t="inlineStr">
+      <c r="S2" t="inlineStr">
         <is>
           <t>ON</t>
         </is>
       </c>
-      <c r="S2" t="inlineStr">
+      <c r="T2" t="inlineStr">
         <is>
           <t>ON</t>
         </is>
       </c>
-      <c r="T2" t="inlineStr">
+      <c r="U2" t="inlineStr">
         <is>
           <t>ON</t>
         </is>
       </c>
-      <c r="U2" t="inlineStr">
+      <c r="V2" t="inlineStr">
         <is>
           <t>ON</t>
         </is>
       </c>
-      <c r="V2" t="inlineStr">
+      <c r="W2" t="inlineStr">
         <is>
           <t>ON</t>
         </is>
       </c>
-      <c r="W2" t="inlineStr">
+      <c r="X2" t="inlineStr">
         <is>
           <t>ON</t>
         </is>
       </c>
-      <c r="X2" t="inlineStr">
+      <c r="Y2" t="inlineStr">
         <is>
           <t>ON</t>
         </is>
       </c>
-      <c r="Y2" t="inlineStr">
+      <c r="Z2" t="inlineStr">
         <is>
           <t>ON</t>
         </is>
       </c>
-      <c r="Z2" t="inlineStr">
+      <c r="AA2" t="inlineStr">
         <is>
           <t>ON</t>
         </is>
       </c>
-      <c r="AA2" t="inlineStr">
+      <c r="AB2" t="inlineStr">
         <is>
           <t>ON</t>
         </is>
       </c>
-      <c r="AB2" t="inlineStr">
+      <c r="AC2" t="inlineStr">
         <is>
           <t>ON</t>
         </is>
@@ -1505,85 +1526,90 @@
       </c>
       <c r="L3" t="inlineStr">
         <is>
+          <t>BOTH</t>
+        </is>
+      </c>
+      <c r="M3" t="inlineStr">
+        <is>
           <t>LEARN_MORE</t>
         </is>
       </c>
-      <c r="M3" t="inlineStr">
+      <c r="N3" t="inlineStr">
         <is>
           <t>CALL</t>
         </is>
       </c>
-      <c r="N3" t="inlineStr">
+      <c r="O3" t="inlineStr">
         <is>
           <t>OFF</t>
         </is>
       </c>
-      <c r="O3" t="inlineStr">
+      <c r="P3" t="inlineStr">
         <is>
           <t>OFF</t>
         </is>
       </c>
-      <c r="P3" t="inlineStr">
+      <c r="Q3" t="inlineStr">
         <is>
           <t>OFF</t>
         </is>
       </c>
-      <c r="Q3" t="inlineStr">
+      <c r="R3" t="inlineStr">
         <is>
           <t>OFF</t>
         </is>
       </c>
-      <c r="R3" t="inlineStr">
+      <c r="S3" t="inlineStr">
         <is>
           <t>OFF</t>
         </is>
       </c>
-      <c r="S3" t="inlineStr">
+      <c r="T3" t="inlineStr">
         <is>
           <t>OFF</t>
         </is>
       </c>
-      <c r="T3" t="inlineStr">
+      <c r="U3" t="inlineStr">
         <is>
           <t>OFF</t>
         </is>
       </c>
-      <c r="U3" t="inlineStr">
+      <c r="V3" t="inlineStr">
         <is>
           <t>OFF</t>
         </is>
       </c>
-      <c r="V3" t="inlineStr">
+      <c r="W3" t="inlineStr">
         <is>
           <t>OFF</t>
         </is>
       </c>
-      <c r="W3" t="inlineStr">
+      <c r="X3" t="inlineStr">
         <is>
           <t>OFF</t>
         </is>
       </c>
-      <c r="X3" t="inlineStr">
+      <c r="Y3" t="inlineStr">
         <is>
           <t>OFF</t>
         </is>
       </c>
-      <c r="Y3" t="inlineStr">
+      <c r="Z3" t="inlineStr">
         <is>
           <t>OFF</t>
         </is>
       </c>
-      <c r="Z3" t="inlineStr">
+      <c r="AA3" t="inlineStr">
         <is>
           <t>OFF</t>
         </is>
       </c>
-      <c r="AA3" t="inlineStr">
+      <c r="AB3" t="inlineStr">
         <is>
           <t>OFF</t>
         </is>
       </c>
-      <c r="AB3" t="inlineStr">
+      <c r="AC3" t="inlineStr">
         <is>
           <t>OFF</t>
         </is>
@@ -1637,10 +1663,15 @@
       </c>
       <c r="L4" t="inlineStr">
         <is>
+          <t>FIRST_ONLY</t>
+        </is>
+      </c>
+      <c r="M4" t="inlineStr">
+        <is>
           <t>SIGN_UP</t>
         </is>
       </c>
-      <c r="M4" t="inlineStr">
+      <c r="N4" t="inlineStr">
         <is>
           <t>MESSENGER</t>
         </is>
@@ -1687,12 +1718,12 @@
           <t>ADD_TO_CART</t>
         </is>
       </c>
-      <c r="L5" t="inlineStr">
+      <c r="M5" t="inlineStr">
         <is>
           <t>SUBSCRIBE</t>
         </is>
       </c>
-      <c r="M5" t="inlineStr">
+      <c r="N5" t="inlineStr">
         <is>
           <t>WHATSAPP</t>
         </is>
@@ -1729,7 +1760,7 @@
           <t>INITIATE_CHECKOUT</t>
         </is>
       </c>
-      <c r="L6" t="inlineStr">
+      <c r="M6" t="inlineStr">
         <is>
           <t>DOWNLOAD</t>
         </is>
@@ -1761,7 +1792,7 @@
           <t>ADD_PAYMENT_INFO</t>
         </is>
       </c>
-      <c r="L7" t="inlineStr">
+      <c r="M7" t="inlineStr">
         <is>
           <t>BOOK_TRAVEL</t>
         </is>
@@ -1788,7 +1819,7 @@
           <t>VIEW_CONTENT</t>
         </is>
       </c>
-      <c r="L8" t="inlineStr">
+      <c r="M8" t="inlineStr">
         <is>
           <t>CONTACT_US</t>
         </is>
@@ -1810,7 +1841,7 @@
           <t>SEARCH</t>
         </is>
       </c>
-      <c r="L9" t="inlineStr">
+      <c r="M9" t="inlineStr">
         <is>
           <t>GET_OFFER</t>
         </is>
@@ -1832,7 +1863,7 @@
           <t>SUBSCRIBE</t>
         </is>
       </c>
-      <c r="L10" t="inlineStr">
+      <c r="M10" t="inlineStr">
         <is>
           <t>GET_QUOTE</t>
         </is>
@@ -1854,7 +1885,7 @@
           <t>CONTACT</t>
         </is>
       </c>
-      <c r="L11" t="inlineStr">
+      <c r="M11" t="inlineStr">
         <is>
           <t>APPLY_NOW</t>
         </is>
@@ -1876,7 +1907,7 @@
           <t>DONATE</t>
         </is>
       </c>
-      <c r="L12" t="inlineStr">
+      <c r="M12" t="inlineStr">
         <is>
           <t>ORDER_NOW</t>
         </is>
@@ -1898,7 +1929,7 @@
           <t>OTHER</t>
         </is>
       </c>
-      <c r="L13" t="inlineStr">
+      <c r="M13" t="inlineStr">
         <is>
           <t>DONATE_NOW</t>
         </is>
@@ -1910,7 +1941,7 @@
           <t>CONVERSATIONS</t>
         </is>
       </c>
-      <c r="L14" t="inlineStr">
+      <c r="M14" t="inlineStr">
         <is>
           <t>INSTALL_APP</t>
         </is>
@@ -1922,7 +1953,7 @@
           <t>APP_INSTALLS</t>
         </is>
       </c>
-      <c r="L15" t="inlineStr">
+      <c r="M15" t="inlineStr">
         <is>
           <t>USE_APP</t>
         </is>
@@ -1934,49 +1965,49 @@
           <t>AD_RECALL_LIFT</t>
         </is>
       </c>
-      <c r="L16" t="inlineStr">
+      <c r="M16" t="inlineStr">
         <is>
           <t>WATCH_MORE</t>
         </is>
       </c>
     </row>
     <row r="17">
-      <c r="L17" t="inlineStr">
+      <c r="M17" t="inlineStr">
         <is>
           <t>LISTEN_NOW</t>
         </is>
       </c>
     </row>
     <row r="18">
-      <c r="L18" t="inlineStr">
+      <c r="M18" t="inlineStr">
         <is>
           <t>SEND_MESSAGE</t>
         </is>
       </c>
     </row>
     <row r="19">
-      <c r="L19" t="inlineStr">
+      <c r="M19" t="inlineStr">
         <is>
           <t>MESSAGE_PAGE</t>
         </is>
       </c>
     </row>
     <row r="20">
-      <c r="L20" t="inlineStr">
+      <c r="M20" t="inlineStr">
         <is>
           <t>GET_DIRECTIONS</t>
         </is>
       </c>
     </row>
     <row r="21">
-      <c r="L21" t="inlineStr">
+      <c r="M21" t="inlineStr">
         <is>
           <t>CALL_NOW</t>
         </is>
       </c>
     </row>
     <row r="22">
-      <c r="L22" t="inlineStr">
+      <c r="M22" t="inlineStr">
         <is>
           <t>NO_BUTTON</t>
         </is>

</xml_diff>

<commit_message>
Keep all 14 adv_* columns; skip UI-only ones at upload with a note
User wants the template to mirror Ads Manager's full Advantage+
creative section, so all 14 toggles stay as columns. At upload time
the script only forwards the 7 keys the Marketing API actually
accepts (IG_VIDEO_NATIVE_SUBTITLE, IMAGE_ANIMATION, PROFILE_CARD,
TEXT_OVERLAY_TRANSLATION, plus 3 catalog-only ones). The other 10
columns map to UI-only Ads Manager toggles that Meta doesn't expose
in the API — they're silently skipped at upload, with a one-line
note listing which were skipped so the user knows to configure
those manually in Ads Manager after upload.
</commit_message>
<xml_diff>
--- a/template.xlsx
+++ b/template.xlsx
@@ -26,13 +26,23 @@
     <definedName name="cta_options">'_options'!$M$2:$M$22</definedName>
     <definedName name="browser_addon_options">'_options'!$N$2:$N$5</definedName>
     <definedName name="advantage_plus_creative_options">'_options'!$O$2:$O$3</definedName>
-    <definedName name="adv_ig_video_subtitle_options">'_options'!$P$2:$P$3</definedName>
-    <definedName name="adv_image_animation_options">'_options'!$Q$2:$Q$3</definedName>
-    <definedName name="adv_profile_card_options">'_options'!$R$2:$R$3</definedName>
-    <definedName name="adv_text_overlay_translation_options">'_options'!$S$2:$S$3</definedName>
-    <definedName name="adv_product_browsing_options">'_options'!$T$2:$T$3</definedName>
-    <definedName name="adv_product_metadata_options">'_options'!$U$2:$U$3</definedName>
-    <definedName name="adv_catalog_enhancements_options">'_options'!$V$2:$V$3</definedName>
+    <definedName name="adv_add_overlays_options">'_options'!$P$2:$P$3</definedName>
+    <definedName name="adv_image_touchups_options">'_options'!$Q$2:$Q$3</definedName>
+    <definedName name="adv_music_options">'_options'!$R$2:$R$3</definedName>
+    <definedName name="adv_text_generation_options">'_options'!$S$2:$S$3</definedName>
+    <definedName name="adv_image_animation_options">'_options'!$T$2:$T$3</definedName>
+    <definedName name="adv_product_tags_options">'_options'!$U$2:$U$3</definedName>
+    <definedName name="adv_relevant_comments_options">'_options'!$V$2:$V$3</definedName>
+    <definedName name="adv_enhance_cta_options">'_options'!$W$2:$W$3</definedName>
+    <definedName name="adv_brightness_contrast_options">'_options'!$X$2:$X$3</definedName>
+    <definedName name="adv_reveal_details_options">'_options'!$Y$2:$Y$3</definedName>
+    <definedName name="adv_spotlights_options">'_options'!$Z$2:$Z$3</definedName>
+    <definedName name="adv_text_overlay_translation_options">'_options'!$AA$2:$AA$3</definedName>
+    <definedName name="adv_ig_video_subtitle_options">'_options'!$AB$2:$AB$3</definedName>
+    <definedName name="adv_profile_card_options">'_options'!$AC$2:$AC$3</definedName>
+    <definedName name="adv_product_browsing_options">'_options'!$AD$2:$AD$3</definedName>
+    <definedName name="adv_product_metadata_options">'_options'!$AE$2:$AE$3</definedName>
+    <definedName name="adv_catalog_enhancements_options">'_options'!$AF$2:$AF$3</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -437,7 +447,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:BQ2"/>
+  <dimension ref="A1:CA2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -502,13 +512,23 @@
     <col width="14" customWidth="1" min="60" max="60"/>
     <col width="19" customWidth="1" min="61" max="61"/>
     <col width="25" customWidth="1" min="62" max="62"/>
-    <col width="23" customWidth="1" min="63" max="63"/>
-    <col width="21" customWidth="1" min="64" max="64"/>
-    <col width="18" customWidth="1" min="65" max="65"/>
-    <col width="30" customWidth="1" min="66" max="66"/>
-    <col width="22" customWidth="1" min="67" max="67"/>
-    <col width="22" customWidth="1" min="68" max="68"/>
-    <col width="26" customWidth="1" min="69" max="69"/>
+    <col width="18" customWidth="1" min="63" max="63"/>
+    <col width="20" customWidth="1" min="64" max="64"/>
+    <col width="14" customWidth="1" min="65" max="65"/>
+    <col width="21" customWidth="1" min="66" max="66"/>
+    <col width="21" customWidth="1" min="67" max="67"/>
+    <col width="18" customWidth="1" min="68" max="68"/>
+    <col width="23" customWidth="1" min="69" max="69"/>
+    <col width="17" customWidth="1" min="70" max="70"/>
+    <col width="25" customWidth="1" min="71" max="71"/>
+    <col width="20" customWidth="1" min="72" max="72"/>
+    <col width="16" customWidth="1" min="73" max="73"/>
+    <col width="30" customWidth="1" min="74" max="74"/>
+    <col width="23" customWidth="1" min="75" max="75"/>
+    <col width="18" customWidth="1" min="76" max="76"/>
+    <col width="22" customWidth="1" min="77" max="77"/>
+    <col width="22" customWidth="1" min="78" max="78"/>
+    <col width="26" customWidth="1" min="79" max="79"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -824,35 +844,85 @@
       </c>
       <c r="BK1" t="inlineStr">
         <is>
+          <t>adv_add_overlays</t>
+        </is>
+      </c>
+      <c r="BL1" t="inlineStr">
+        <is>
+          <t>adv_image_touchups</t>
+        </is>
+      </c>
+      <c r="BM1" t="inlineStr">
+        <is>
+          <t>adv_music</t>
+        </is>
+      </c>
+      <c r="BN1" t="inlineStr">
+        <is>
+          <t>adv_text_generation</t>
+        </is>
+      </c>
+      <c r="BO1" t="inlineStr">
+        <is>
+          <t>adv_image_animation</t>
+        </is>
+      </c>
+      <c r="BP1" t="inlineStr">
+        <is>
+          <t>adv_product_tags</t>
+        </is>
+      </c>
+      <c r="BQ1" t="inlineStr">
+        <is>
+          <t>adv_relevant_comments</t>
+        </is>
+      </c>
+      <c r="BR1" t="inlineStr">
+        <is>
+          <t>adv_enhance_cta</t>
+        </is>
+      </c>
+      <c r="BS1" t="inlineStr">
+        <is>
+          <t>adv_brightness_contrast</t>
+        </is>
+      </c>
+      <c r="BT1" t="inlineStr">
+        <is>
+          <t>adv_reveal_details</t>
+        </is>
+      </c>
+      <c r="BU1" t="inlineStr">
+        <is>
+          <t>adv_spotlights</t>
+        </is>
+      </c>
+      <c r="BV1" t="inlineStr">
+        <is>
+          <t>adv_text_overlay_translation</t>
+        </is>
+      </c>
+      <c r="BW1" t="inlineStr">
+        <is>
           <t>adv_ig_video_subtitle</t>
         </is>
       </c>
-      <c r="BL1" t="inlineStr">
-        <is>
-          <t>adv_image_animation</t>
-        </is>
-      </c>
-      <c r="BM1" t="inlineStr">
+      <c r="BX1" t="inlineStr">
         <is>
           <t>adv_profile_card</t>
         </is>
       </c>
-      <c r="BN1" t="inlineStr">
-        <is>
-          <t>adv_text_overlay_translation</t>
-        </is>
-      </c>
-      <c r="BO1" t="inlineStr">
+      <c r="BY1" t="inlineStr">
         <is>
           <t>adv_product_browsing</t>
         </is>
       </c>
-      <c r="BP1" t="inlineStr">
+      <c r="BZ1" t="inlineStr">
         <is>
           <t>adv_product_metadata</t>
         </is>
       </c>
-      <c r="BQ1" t="inlineStr">
+      <c r="CA1" t="inlineStr">
         <is>
           <t>adv_catalog_enhancements</t>
         </is>
@@ -1014,9 +1084,19 @@
       <c r="BO2" t="inlineStr"/>
       <c r="BP2" t="inlineStr"/>
       <c r="BQ2" t="inlineStr"/>
+      <c r="BR2" t="inlineStr"/>
+      <c r="BS2" t="inlineStr"/>
+      <c r="BT2" t="inlineStr"/>
+      <c r="BU2" t="inlineStr"/>
+      <c r="BV2" t="inlineStr"/>
+      <c r="BW2" t="inlineStr"/>
+      <c r="BX2" t="inlineStr"/>
+      <c r="BY2" t="inlineStr"/>
+      <c r="BZ2" t="inlineStr"/>
+      <c r="CA2" t="inlineStr"/>
     </row>
   </sheetData>
-  <dataValidations count="22">
+  <dataValidations count="32">
     <dataValidation sqref="C2:C500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid value" error="Pick a valid campaign_objective" promptTitle="campaign_objective" prompt="Choose from the list" type="list">
       <formula1>campaign_objective_options</formula1>
     </dataValidation>
@@ -1062,25 +1142,55 @@
     <dataValidation sqref="BJ2:BJ500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid value" error="Pick a valid advantage_plus_creative" promptTitle="advantage_plus_creative" prompt="Choose from the list" type="list">
       <formula1>advantage_plus_creative_options</formula1>
     </dataValidation>
-    <dataValidation sqref="BK2:BK500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid value" error="Pick a valid adv_ig_video_subtitle" promptTitle="adv_ig_video_subtitle" prompt="Choose from the list" type="list">
+    <dataValidation sqref="BK2:BK500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid value" error="Pick a valid adv_add_overlays" promptTitle="adv_add_overlays" prompt="Choose from the list" type="list">
+      <formula1>adv_add_overlays_options</formula1>
+    </dataValidation>
+    <dataValidation sqref="BL2:BL500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid value" error="Pick a valid adv_image_touchups" promptTitle="adv_image_touchups" prompt="Choose from the list" type="list">
+      <formula1>adv_image_touchups_options</formula1>
+    </dataValidation>
+    <dataValidation sqref="BM2:BM500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid value" error="Pick a valid adv_music" promptTitle="adv_music" prompt="Choose from the list" type="list">
+      <formula1>adv_music_options</formula1>
+    </dataValidation>
+    <dataValidation sqref="BN2:BN500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid value" error="Pick a valid adv_text_generation" promptTitle="adv_text_generation" prompt="Choose from the list" type="list">
+      <formula1>adv_text_generation_options</formula1>
+    </dataValidation>
+    <dataValidation sqref="BO2:BO500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid value" error="Pick a valid adv_image_animation" promptTitle="adv_image_animation" prompt="Choose from the list" type="list">
+      <formula1>adv_image_animation_options</formula1>
+    </dataValidation>
+    <dataValidation sqref="BP2:BP500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid value" error="Pick a valid adv_product_tags" promptTitle="adv_product_tags" prompt="Choose from the list" type="list">
+      <formula1>adv_product_tags_options</formula1>
+    </dataValidation>
+    <dataValidation sqref="BQ2:BQ500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid value" error="Pick a valid adv_relevant_comments" promptTitle="adv_relevant_comments" prompt="Choose from the list" type="list">
+      <formula1>adv_relevant_comments_options</formula1>
+    </dataValidation>
+    <dataValidation sqref="BR2:BR500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid value" error="Pick a valid adv_enhance_cta" promptTitle="adv_enhance_cta" prompt="Choose from the list" type="list">
+      <formula1>adv_enhance_cta_options</formula1>
+    </dataValidation>
+    <dataValidation sqref="BS2:BS500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid value" error="Pick a valid adv_brightness_contrast" promptTitle="adv_brightness_contrast" prompt="Choose from the list" type="list">
+      <formula1>adv_brightness_contrast_options</formula1>
+    </dataValidation>
+    <dataValidation sqref="BT2:BT500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid value" error="Pick a valid adv_reveal_details" promptTitle="adv_reveal_details" prompt="Choose from the list" type="list">
+      <formula1>adv_reveal_details_options</formula1>
+    </dataValidation>
+    <dataValidation sqref="BU2:BU500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid value" error="Pick a valid adv_spotlights" promptTitle="adv_spotlights" prompt="Choose from the list" type="list">
+      <formula1>adv_spotlights_options</formula1>
+    </dataValidation>
+    <dataValidation sqref="BV2:BV500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid value" error="Pick a valid adv_text_overlay_translation" promptTitle="adv_text_overlay_translation" prompt="Choose from the list" type="list">
+      <formula1>adv_text_overlay_translation_options</formula1>
+    </dataValidation>
+    <dataValidation sqref="BW2:BW500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid value" error="Pick a valid adv_ig_video_subtitle" promptTitle="adv_ig_video_subtitle" prompt="Choose from the list" type="list">
       <formula1>adv_ig_video_subtitle_options</formula1>
     </dataValidation>
-    <dataValidation sqref="BL2:BL500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid value" error="Pick a valid adv_image_animation" promptTitle="adv_image_animation" prompt="Choose from the list" type="list">
-      <formula1>adv_image_animation_options</formula1>
-    </dataValidation>
-    <dataValidation sqref="BM2:BM500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid value" error="Pick a valid adv_profile_card" promptTitle="adv_profile_card" prompt="Choose from the list" type="list">
+    <dataValidation sqref="BX2:BX500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid value" error="Pick a valid adv_profile_card" promptTitle="adv_profile_card" prompt="Choose from the list" type="list">
       <formula1>adv_profile_card_options</formula1>
     </dataValidation>
-    <dataValidation sqref="BN2:BN500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid value" error="Pick a valid adv_text_overlay_translation" promptTitle="adv_text_overlay_translation" prompt="Choose from the list" type="list">
-      <formula1>adv_text_overlay_translation_options</formula1>
-    </dataValidation>
-    <dataValidation sqref="BO2:BO500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid value" error="Pick a valid adv_product_browsing" promptTitle="adv_product_browsing" prompt="Choose from the list" type="list">
+    <dataValidation sqref="BY2:BY500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid value" error="Pick a valid adv_product_browsing" promptTitle="adv_product_browsing" prompt="Choose from the list" type="list">
       <formula1>adv_product_browsing_options</formula1>
     </dataValidation>
-    <dataValidation sqref="BP2:BP500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid value" error="Pick a valid adv_product_metadata" promptTitle="adv_product_metadata" prompt="Choose from the list" type="list">
+    <dataValidation sqref="BZ2:BZ500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid value" error="Pick a valid adv_product_metadata" promptTitle="adv_product_metadata" prompt="Choose from the list" type="list">
       <formula1>adv_product_metadata_options</formula1>
     </dataValidation>
-    <dataValidation sqref="BQ2:BQ500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid value" error="Pick a valid adv_catalog_enhancements" promptTitle="adv_catalog_enhancements" prompt="Choose from the list" type="list">
+    <dataValidation sqref="CA2:CA500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid value" error="Pick a valid adv_catalog_enhancements" promptTitle="adv_catalog_enhancements" prompt="Choose from the list" type="list">
       <formula1>adv_catalog_enhancements_options</formula1>
     </dataValidation>
   </dataValidations>
@@ -1094,7 +1204,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:V22"/>
+  <dimension ref="A1:AF22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1175,35 +1285,85 @@
       </c>
       <c r="P1" t="inlineStr">
         <is>
+          <t>adv_add_overlays</t>
+        </is>
+      </c>
+      <c r="Q1" t="inlineStr">
+        <is>
+          <t>adv_image_touchups</t>
+        </is>
+      </c>
+      <c r="R1" t="inlineStr">
+        <is>
+          <t>adv_music</t>
+        </is>
+      </c>
+      <c r="S1" t="inlineStr">
+        <is>
+          <t>adv_text_generation</t>
+        </is>
+      </c>
+      <c r="T1" t="inlineStr">
+        <is>
+          <t>adv_image_animation</t>
+        </is>
+      </c>
+      <c r="U1" t="inlineStr">
+        <is>
+          <t>adv_product_tags</t>
+        </is>
+      </c>
+      <c r="V1" t="inlineStr">
+        <is>
+          <t>adv_relevant_comments</t>
+        </is>
+      </c>
+      <c r="W1" t="inlineStr">
+        <is>
+          <t>adv_enhance_cta</t>
+        </is>
+      </c>
+      <c r="X1" t="inlineStr">
+        <is>
+          <t>adv_brightness_contrast</t>
+        </is>
+      </c>
+      <c r="Y1" t="inlineStr">
+        <is>
+          <t>adv_reveal_details</t>
+        </is>
+      </c>
+      <c r="Z1" t="inlineStr">
+        <is>
+          <t>adv_spotlights</t>
+        </is>
+      </c>
+      <c r="AA1" t="inlineStr">
+        <is>
+          <t>adv_text_overlay_translation</t>
+        </is>
+      </c>
+      <c r="AB1" t="inlineStr">
+        <is>
           <t>adv_ig_video_subtitle</t>
         </is>
       </c>
-      <c r="Q1" t="inlineStr">
-        <is>
-          <t>adv_image_animation</t>
-        </is>
-      </c>
-      <c r="R1" t="inlineStr">
+      <c r="AC1" t="inlineStr">
         <is>
           <t>adv_profile_card</t>
         </is>
       </c>
-      <c r="S1" t="inlineStr">
-        <is>
-          <t>adv_text_overlay_translation</t>
-        </is>
-      </c>
-      <c r="T1" t="inlineStr">
+      <c r="AD1" t="inlineStr">
         <is>
           <t>adv_product_browsing</t>
         </is>
       </c>
-      <c r="U1" t="inlineStr">
+      <c r="AE1" t="inlineStr">
         <is>
           <t>adv_product_metadata</t>
         </is>
       </c>
-      <c r="V1" t="inlineStr">
+      <c r="AF1" t="inlineStr">
         <is>
           <t>adv_catalog_enhancements</t>
         </is>
@@ -1320,6 +1480,56 @@
           <t>ON</t>
         </is>
       </c>
+      <c r="W2" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+      <c r="X2" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+      <c r="Y2" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+      <c r="Z2" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+      <c r="AA2" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+      <c r="AB2" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+      <c r="AC2" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+      <c r="AD2" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+      <c r="AE2" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+      <c r="AF2" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -1428,6 +1638,56 @@
         </is>
       </c>
       <c r="V3" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+      <c r="W3" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+      <c r="X3" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+      <c r="Y3" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+      <c r="Z3" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+      <c r="AA3" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+      <c r="AB3" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+      <c r="AC3" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+      <c r="AD3" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+      <c r="AE3" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+      <c r="AF3" t="inlineStr">
         <is>
           <t>OFF</t>
         </is>

</xml_diff>